<commit_message>
REIMPORTING DAY YARD LPOS
</commit_message>
<xml_diff>
--- a/dar yard lpos.xlsx
+++ b/dar yard lpos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tungsten\Documents\Backup from old pc\WINDOWS 11\Fuel_Order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DCC6C2-6C69-413D-9087-4279B27141C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5297E8AE-EC1C-4A2B-8686-1BB0BD8B0A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{644A8DE3-68DC-4C6A-A18C-611A87002412}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="5" xr2:uid="{644A8DE3-68DC-4C6A-A18C-611A87002412}"/>
   </bookViews>
   <sheets>
     <sheet name="JAN" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="MAR" sheetId="3" r:id="rId3"/>
     <sheet name="APR" sheetId="4" r:id="rId4"/>
     <sheet name="MAY" sheetId="5" r:id="rId5"/>
+    <sheet name="JUN" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1167" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1404" uniqueCount="538">
   <si>
     <t>DATE</t>
   </si>
@@ -1523,6 +1524,135 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>T958 EQM</t>
+  </si>
+  <si>
+    <t>T231 EQL</t>
+  </si>
+  <si>
+    <t>T957 EQM</t>
+  </si>
+  <si>
+    <t>T281 EQL</t>
+  </si>
+  <si>
+    <t>T484 EEQ</t>
+  </si>
+  <si>
+    <t>T665 ECQ</t>
+  </si>
+  <si>
+    <t>T571 EQF</t>
+  </si>
+  <si>
+    <t>T593 DRE</t>
+  </si>
+  <si>
+    <t>T358 EQF</t>
+  </si>
+  <si>
+    <t>T147 DZY</t>
+  </si>
+  <si>
+    <t>T717 EQD</t>
+  </si>
+  <si>
+    <t>T113 DVL</t>
+  </si>
+  <si>
+    <t>T459 EAG</t>
+  </si>
+  <si>
+    <t>T580 DRE</t>
+  </si>
+  <si>
+    <t>T595 DRE</t>
+  </si>
+  <si>
+    <t>T651 ECQ</t>
+  </si>
+  <si>
+    <t>T355 EQF</t>
+  </si>
+  <si>
+    <t>T681 EAQ</t>
+  </si>
+  <si>
+    <t>T278 EQL</t>
+  </si>
+  <si>
+    <t>T272 EQL</t>
+  </si>
+  <si>
+    <t>T529 DRE</t>
+  </si>
+  <si>
+    <t>T282 EQL</t>
+  </si>
+  <si>
+    <t>T192 CHM</t>
+  </si>
+  <si>
+    <t>T660 ECQ</t>
+  </si>
+  <si>
+    <t>T521 DRF</t>
+  </si>
+  <si>
+    <t>T594 DRE</t>
+  </si>
+  <si>
+    <t>T840 DNH</t>
+  </si>
+  <si>
+    <t>T158 DZY</t>
+  </si>
+  <si>
+    <t>T143 DRF</t>
+  </si>
+  <si>
+    <t>T602 EAG</t>
+  </si>
+  <si>
+    <t>T516 EQL</t>
+  </si>
+  <si>
+    <t>T280 EQL</t>
+  </si>
+  <si>
+    <t>T156 EQL</t>
+  </si>
+  <si>
+    <t>T163 EQL</t>
+  </si>
+  <si>
+    <t>T221 EQL</t>
+  </si>
+  <si>
+    <t>T632 EQD</t>
+  </si>
+  <si>
+    <t>T123 DYY</t>
+  </si>
+  <si>
+    <t>T160 EQL</t>
+  </si>
+  <si>
+    <t>T125 DYY</t>
+  </si>
+  <si>
+    <t>T165 EGJ</t>
+  </si>
+  <si>
+    <t>KDV 941D</t>
+  </si>
+  <si>
+    <t>T644 EAF</t>
+  </si>
+  <si>
+    <t>T130 EFP</t>
   </si>
 </sst>
 </file>
@@ -1873,7 +2003,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1981,6 +2111,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16414,7 +16545,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC24F6D-C424-46A9-9BEA-CF11769827F8}">
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E253"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.44140625" style="6" bestFit="1" customWidth="1"/>
@@ -19574,7 +19705,7 @@
         <v>3840</v>
       </c>
       <c r="E196">
-        <f t="shared" ref="E196:E232" si="3">C196*D196</f>
+        <f t="shared" ref="E196:E253" si="3">C196*D196</f>
         <v>2265600</v>
       </c>
     </row>
@@ -20160,6 +20291,3631 @@
         <v>384000</v>
       </c>
     </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A233" s="37">
+        <v>46172</v>
+      </c>
+      <c r="B233" t="s">
+        <v>495</v>
+      </c>
+      <c r="C233">
+        <v>20</v>
+      </c>
+      <c r="D233">
+        <v>4330</v>
+      </c>
+      <c r="E233">
+        <f t="shared" si="3"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B234" t="s">
+        <v>496</v>
+      </c>
+      <c r="C234">
+        <v>20</v>
+      </c>
+      <c r="D234">
+        <v>4330</v>
+      </c>
+      <c r="E234">
+        <f t="shared" si="3"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B235" t="s">
+        <v>88</v>
+      </c>
+      <c r="C235">
+        <v>40</v>
+      </c>
+      <c r="D235">
+        <v>4330</v>
+      </c>
+      <c r="E235">
+        <f t="shared" si="3"/>
+        <v>173200</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B236" t="s">
+        <v>17</v>
+      </c>
+      <c r="C236">
+        <v>10</v>
+      </c>
+      <c r="D236">
+        <v>4330</v>
+      </c>
+      <c r="E236">
+        <f t="shared" si="3"/>
+        <v>43300</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B237" t="s">
+        <v>23</v>
+      </c>
+      <c r="C237">
+        <v>538</v>
+      </c>
+      <c r="D237">
+        <v>4330</v>
+      </c>
+      <c r="E237">
+        <f t="shared" si="3"/>
+        <v>2329540</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B238" t="s">
+        <v>29</v>
+      </c>
+      <c r="C238">
+        <v>430</v>
+      </c>
+      <c r="D238">
+        <v>4330</v>
+      </c>
+      <c r="E238">
+        <f t="shared" si="3"/>
+        <v>1861900</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B239" t="s">
+        <v>70</v>
+      </c>
+      <c r="C239">
+        <v>590</v>
+      </c>
+      <c r="D239">
+        <v>4330</v>
+      </c>
+      <c r="E239">
+        <f t="shared" si="3"/>
+        <v>2554700</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B240" t="s">
+        <v>88</v>
+      </c>
+      <c r="C240">
+        <v>430</v>
+      </c>
+      <c r="D240">
+        <v>4330</v>
+      </c>
+      <c r="E240">
+        <f t="shared" si="3"/>
+        <v>1861900</v>
+      </c>
+    </row>
+    <row r="241" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B241" t="s">
+        <v>497</v>
+      </c>
+      <c r="C241">
+        <v>598</v>
+      </c>
+      <c r="D241">
+        <v>4330</v>
+      </c>
+      <c r="E241">
+        <f t="shared" si="3"/>
+        <v>2589340</v>
+      </c>
+    </row>
+    <row r="242" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B242" t="s">
+        <v>51</v>
+      </c>
+      <c r="C242">
+        <v>430</v>
+      </c>
+      <c r="D242">
+        <v>4330</v>
+      </c>
+      <c r="E242">
+        <f t="shared" si="3"/>
+        <v>1861900</v>
+      </c>
+    </row>
+    <row r="243" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B243" t="s">
+        <v>496</v>
+      </c>
+      <c r="C243">
+        <v>600</v>
+      </c>
+      <c r="D243">
+        <v>4330</v>
+      </c>
+      <c r="E243">
+        <f t="shared" si="3"/>
+        <v>2598000</v>
+      </c>
+    </row>
+    <row r="244" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B244" t="s">
+        <v>22</v>
+      </c>
+      <c r="C244">
+        <v>374</v>
+      </c>
+      <c r="D244">
+        <v>4330</v>
+      </c>
+      <c r="E244">
+        <f t="shared" si="3"/>
+        <v>1619420</v>
+      </c>
+    </row>
+    <row r="245" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B245" t="s">
+        <v>498</v>
+      </c>
+      <c r="C245">
+        <v>592</v>
+      </c>
+      <c r="D245">
+        <v>4330</v>
+      </c>
+      <c r="E245">
+        <f t="shared" si="3"/>
+        <v>2563360</v>
+      </c>
+    </row>
+    <row r="246" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B246" t="s">
+        <v>495</v>
+      </c>
+      <c r="C246">
+        <v>596</v>
+      </c>
+      <c r="D246">
+        <v>4330</v>
+      </c>
+      <c r="E246">
+        <f t="shared" si="3"/>
+        <v>2580680</v>
+      </c>
+    </row>
+    <row r="247" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B247" t="s">
+        <v>490</v>
+      </c>
+      <c r="C247">
+        <v>600</v>
+      </c>
+      <c r="D247">
+        <v>4330</v>
+      </c>
+      <c r="E247">
+        <f t="shared" si="3"/>
+        <v>2598000</v>
+      </c>
+    </row>
+    <row r="248" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B248" t="s">
+        <v>3</v>
+      </c>
+      <c r="C248">
+        <v>130</v>
+      </c>
+      <c r="D248">
+        <v>4330</v>
+      </c>
+      <c r="E248">
+        <f t="shared" si="3"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="249" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B249" t="s">
+        <v>16</v>
+      </c>
+      <c r="C249">
+        <v>130</v>
+      </c>
+      <c r="D249">
+        <v>4330</v>
+      </c>
+      <c r="E249">
+        <f t="shared" si="3"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="250" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B250" t="s">
+        <v>209</v>
+      </c>
+      <c r="C250">
+        <v>388</v>
+      </c>
+      <c r="D250">
+        <v>4330</v>
+      </c>
+      <c r="E250">
+        <f t="shared" si="3"/>
+        <v>1680040</v>
+      </c>
+    </row>
+    <row r="251" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B251" t="s">
+        <v>49</v>
+      </c>
+      <c r="C251">
+        <v>550</v>
+      </c>
+      <c r="D251">
+        <v>4330</v>
+      </c>
+      <c r="E251">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="252" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B252" t="s">
+        <v>19</v>
+      </c>
+      <c r="C252">
+        <v>130</v>
+      </c>
+      <c r="D252">
+        <v>4330</v>
+      </c>
+      <c r="E252">
+        <f t="shared" si="3"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="253" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B253" t="s">
+        <v>18</v>
+      </c>
+      <c r="C253">
+        <v>342</v>
+      </c>
+      <c r="D253">
+        <v>4330</v>
+      </c>
+      <c r="E253">
+        <f t="shared" si="3"/>
+        <v>1480860</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C60458-4749-4ACB-9FC1-AAB0CFF01868}">
+  <dimension ref="A1:E216"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="37">
+        <v>46174</v>
+      </c>
+      <c r="B1" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1">
+        <v>550</v>
+      </c>
+      <c r="D1">
+        <v>4330</v>
+      </c>
+      <c r="E1">
+        <f t="shared" ref="E1:E64" si="0">C1*D1</f>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>374</v>
+      </c>
+      <c r="C2">
+        <v>550</v>
+      </c>
+      <c r="D2">
+        <v>4330</v>
+      </c>
+      <c r="E2">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>4330</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="0"/>
+        <v>21650</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C4">
+        <v>550</v>
+      </c>
+      <c r="D4">
+        <v>4330</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5">
+        <v>550</v>
+      </c>
+      <c r="D5">
+        <v>4330</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C6">
+        <v>550</v>
+      </c>
+      <c r="D6">
+        <v>4330</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>501</v>
+      </c>
+      <c r="C7">
+        <v>550</v>
+      </c>
+      <c r="D7">
+        <v>4330</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>502</v>
+      </c>
+      <c r="C8">
+        <v>550</v>
+      </c>
+      <c r="D8">
+        <v>4330</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9">
+        <v>531</v>
+      </c>
+      <c r="D9">
+        <v>4330</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>2299230</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>503</v>
+      </c>
+      <c r="C10">
+        <v>573</v>
+      </c>
+      <c r="D10">
+        <v>4330</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>2481090</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>504</v>
+      </c>
+      <c r="C11">
+        <v>550</v>
+      </c>
+      <c r="D11">
+        <v>4330</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>323</v>
+      </c>
+      <c r="C12">
+        <v>550</v>
+      </c>
+      <c r="D12">
+        <v>4330</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13">
+        <v>550</v>
+      </c>
+      <c r="D13">
+        <v>4330</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>505</v>
+      </c>
+      <c r="C14">
+        <v>550</v>
+      </c>
+      <c r="D14">
+        <v>4330</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>334</v>
+      </c>
+      <c r="C15">
+        <v>550</v>
+      </c>
+      <c r="D15">
+        <v>4330</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16">
+        <v>345</v>
+      </c>
+      <c r="D16">
+        <v>4330</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>1493850</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>293</v>
+      </c>
+      <c r="C17">
+        <v>550</v>
+      </c>
+      <c r="D17">
+        <v>4330</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>380</v>
+      </c>
+      <c r="C18">
+        <v>550</v>
+      </c>
+      <c r="D18">
+        <v>4330</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>506</v>
+      </c>
+      <c r="C19">
+        <v>517</v>
+      </c>
+      <c r="D19">
+        <v>4330</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>2238610</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>130</v>
+      </c>
+      <c r="D20">
+        <v>4330</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>130</v>
+      </c>
+      <c r="D21">
+        <v>4330</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="37">
+        <v>46175</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22">
+        <v>370</v>
+      </c>
+      <c r="D22">
+        <v>4330</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>1602100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>371</v>
+      </c>
+      <c r="C23">
+        <v>570</v>
+      </c>
+      <c r="D23">
+        <v>4330</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24">
+        <v>523</v>
+      </c>
+      <c r="D24">
+        <v>4330</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="0"/>
+        <v>2264590</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>507</v>
+      </c>
+      <c r="C25">
+        <v>590</v>
+      </c>
+      <c r="D25">
+        <v>4330</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>2554700</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26">
+        <v>370</v>
+      </c>
+      <c r="D26">
+        <v>4330</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>1602100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>508</v>
+      </c>
+      <c r="C27">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>4330</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="0"/>
+        <v>21650</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28">
+        <v>338</v>
+      </c>
+      <c r="D28">
+        <v>4330</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="0"/>
+        <v>1463540</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>509</v>
+      </c>
+      <c r="C29">
+        <v>550</v>
+      </c>
+      <c r="D29">
+        <v>4330</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>251</v>
+      </c>
+      <c r="C30">
+        <v>540</v>
+      </c>
+      <c r="D30">
+        <v>4330</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="0"/>
+        <v>2338200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31">
+        <v>130</v>
+      </c>
+      <c r="D31">
+        <v>4330</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32">
+        <v>550</v>
+      </c>
+      <c r="D32">
+        <v>4330</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="37">
+        <v>46176</v>
+      </c>
+      <c r="B33" t="s">
+        <v>209</v>
+      </c>
+      <c r="C33">
+        <v>370</v>
+      </c>
+      <c r="D33">
+        <v>4330</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="0"/>
+        <v>1602100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34">
+        <v>550</v>
+      </c>
+      <c r="D34">
+        <v>4330</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35">
+        <v>350</v>
+      </c>
+      <c r="D35">
+        <v>4330</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="0"/>
+        <v>1515500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>451</v>
+      </c>
+      <c r="C36">
+        <v>120</v>
+      </c>
+      <c r="D36">
+        <v>4330</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="0"/>
+        <v>519600</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>3</v>
+      </c>
+      <c r="C37">
+        <v>130</v>
+      </c>
+      <c r="D37">
+        <v>4330</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>328</v>
+      </c>
+      <c r="C38">
+        <v>550</v>
+      </c>
+      <c r="D38">
+        <v>4330</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39">
+        <v>580</v>
+      </c>
+      <c r="D39">
+        <v>4330</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="0"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="37">
+        <v>46177</v>
+      </c>
+      <c r="B40" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40">
+        <v>334</v>
+      </c>
+      <c r="D40">
+        <v>4330</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="0"/>
+        <v>1446220</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41">
+        <v>533</v>
+      </c>
+      <c r="D41">
+        <v>4330</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="0"/>
+        <v>2307890</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>510</v>
+      </c>
+      <c r="C42">
+        <v>458</v>
+      </c>
+      <c r="D42">
+        <v>4330</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="0"/>
+        <v>1983140</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B43" t="s">
+        <v>121</v>
+      </c>
+      <c r="C43">
+        <v>20</v>
+      </c>
+      <c r="D43">
+        <v>4330</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="0"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B44" t="s">
+        <v>100</v>
+      </c>
+      <c r="C44">
+        <v>550</v>
+      </c>
+      <c r="D44">
+        <v>4330</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
+        <v>24</v>
+      </c>
+      <c r="C45">
+        <v>5</v>
+      </c>
+      <c r="D45">
+        <v>4330</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="0"/>
+        <v>21650</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B46" t="s">
+        <v>38</v>
+      </c>
+      <c r="C46">
+        <v>550</v>
+      </c>
+      <c r="D46">
+        <v>4330</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>511</v>
+      </c>
+      <c r="C47">
+        <v>575</v>
+      </c>
+      <c r="D47">
+        <v>4330</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="0"/>
+        <v>2489750</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
+        <v>91</v>
+      </c>
+      <c r="C48">
+        <v>550</v>
+      </c>
+      <c r="D48">
+        <v>4330</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B49" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49">
+        <v>130</v>
+      </c>
+      <c r="D49">
+        <v>4330</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B50" t="s">
+        <v>33</v>
+      </c>
+      <c r="C50">
+        <v>20</v>
+      </c>
+      <c r="D50">
+        <v>4330</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="0"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>117</v>
+      </c>
+      <c r="C51">
+        <v>550</v>
+      </c>
+      <c r="D51">
+        <v>4330</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B52" t="s">
+        <v>512</v>
+      </c>
+      <c r="C52">
+        <v>550</v>
+      </c>
+      <c r="D52">
+        <v>4330</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B53" t="s">
+        <v>19</v>
+      </c>
+      <c r="C53">
+        <v>130</v>
+      </c>
+      <c r="D53">
+        <v>4330</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B54" t="s">
+        <v>3</v>
+      </c>
+      <c r="C54">
+        <v>130</v>
+      </c>
+      <c r="D54">
+        <v>4330</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="0"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="37">
+        <v>46178</v>
+      </c>
+      <c r="B55" t="s">
+        <v>513</v>
+      </c>
+      <c r="C55">
+        <v>570</v>
+      </c>
+      <c r="D55">
+        <v>4330</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="0"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B56" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56">
+        <v>570</v>
+      </c>
+      <c r="D56">
+        <v>4330</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="0"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B57" t="s">
+        <v>514</v>
+      </c>
+      <c r="C57">
+        <v>597</v>
+      </c>
+      <c r="D57">
+        <v>4330</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="0"/>
+        <v>2585010</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
+        <v>23</v>
+      </c>
+      <c r="C58">
+        <v>550</v>
+      </c>
+      <c r="D58">
+        <v>4330</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="0"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B59" t="s">
+        <v>94</v>
+      </c>
+      <c r="C59">
+        <v>520</v>
+      </c>
+      <c r="D59">
+        <v>4330</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="0"/>
+        <v>2251600</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>515</v>
+      </c>
+      <c r="C60">
+        <v>20</v>
+      </c>
+      <c r="D60">
+        <v>4330</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="0"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B61" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61">
+        <v>362</v>
+      </c>
+      <c r="D61">
+        <v>4330</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="0"/>
+        <v>1567460</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
+        <v>22</v>
+      </c>
+      <c r="C62">
+        <v>355</v>
+      </c>
+      <c r="D62">
+        <v>4330</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="0"/>
+        <v>1537150</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B63" t="s">
+        <v>87</v>
+      </c>
+      <c r="C63">
+        <v>524</v>
+      </c>
+      <c r="D63">
+        <v>4330</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="0"/>
+        <v>2268920</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
+        <v>26</v>
+      </c>
+      <c r="C64">
+        <v>394</v>
+      </c>
+      <c r="D64">
+        <v>4330</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="0"/>
+        <v>1706020</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" s="37">
+        <v>46179</v>
+      </c>
+      <c r="B65" t="s">
+        <v>49</v>
+      </c>
+      <c r="C65">
+        <v>541</v>
+      </c>
+      <c r="D65">
+        <v>4330</v>
+      </c>
+      <c r="E65">
+        <f t="shared" ref="E65:E128" si="1">C65*D65</f>
+        <v>2342530</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
+        <v>516</v>
+      </c>
+      <c r="C66">
+        <v>575</v>
+      </c>
+      <c r="D66">
+        <v>4330</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="1"/>
+        <v>2489750</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B67" t="s">
+        <v>189</v>
+      </c>
+      <c r="C67">
+        <v>90</v>
+      </c>
+      <c r="D67">
+        <v>4330</v>
+      </c>
+      <c r="E67">
+        <f t="shared" si="1"/>
+        <v>389700</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>508</v>
+      </c>
+      <c r="C68">
+        <v>592</v>
+      </c>
+      <c r="D68">
+        <v>4330</v>
+      </c>
+      <c r="E68">
+        <f t="shared" si="1"/>
+        <v>2563360</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B69" t="s">
+        <v>89</v>
+      </c>
+      <c r="C69">
+        <v>550</v>
+      </c>
+      <c r="D69">
+        <v>4330</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>19</v>
+      </c>
+      <c r="C70">
+        <v>130</v>
+      </c>
+      <c r="D70">
+        <v>4330</v>
+      </c>
+      <c r="E70">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C71">
+        <v>550</v>
+      </c>
+      <c r="D71">
+        <v>4330</v>
+      </c>
+      <c r="E71">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B72" t="s">
+        <v>50</v>
+      </c>
+      <c r="C72">
+        <v>370</v>
+      </c>
+      <c r="D72">
+        <v>4330</v>
+      </c>
+      <c r="E72">
+        <f t="shared" si="1"/>
+        <v>1602100</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B73" t="s">
+        <v>16</v>
+      </c>
+      <c r="C73">
+        <v>130</v>
+      </c>
+      <c r="D73">
+        <v>4330</v>
+      </c>
+      <c r="E73">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B74" t="s">
+        <v>209</v>
+      </c>
+      <c r="C74">
+        <v>406</v>
+      </c>
+      <c r="D74">
+        <v>4330</v>
+      </c>
+      <c r="E74">
+        <f t="shared" si="1"/>
+        <v>1757980</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B75" t="s">
+        <v>18</v>
+      </c>
+      <c r="C75">
+        <v>348</v>
+      </c>
+      <c r="D75">
+        <v>4330</v>
+      </c>
+      <c r="E75">
+        <f t="shared" si="1"/>
+        <v>1506840</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B76" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76">
+        <v>550</v>
+      </c>
+      <c r="D76">
+        <v>4330</v>
+      </c>
+      <c r="E76">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B77" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77">
+        <v>352</v>
+      </c>
+      <c r="D77">
+        <v>4330</v>
+      </c>
+      <c r="E77">
+        <f t="shared" si="1"/>
+        <v>1524160</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B78" t="s">
+        <v>3</v>
+      </c>
+      <c r="C78">
+        <v>130</v>
+      </c>
+      <c r="D78">
+        <v>4330</v>
+      </c>
+      <c r="E78">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B79" t="s">
+        <v>26</v>
+      </c>
+      <c r="C79">
+        <v>386</v>
+      </c>
+      <c r="D79">
+        <v>4330</v>
+      </c>
+      <c r="E79">
+        <f t="shared" si="1"/>
+        <v>1671380</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" s="37">
+        <v>46181</v>
+      </c>
+      <c r="B80" t="s">
+        <v>49</v>
+      </c>
+      <c r="C80">
+        <v>536</v>
+      </c>
+      <c r="D80">
+        <v>4330</v>
+      </c>
+      <c r="E80">
+        <f t="shared" si="1"/>
+        <v>2320880</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B81" t="s">
+        <v>22</v>
+      </c>
+      <c r="C81">
+        <v>344</v>
+      </c>
+      <c r="D81">
+        <v>4330</v>
+      </c>
+      <c r="E81">
+        <f t="shared" si="1"/>
+        <v>1489520</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B82" t="s">
+        <v>517</v>
+      </c>
+      <c r="C82">
+        <v>2</v>
+      </c>
+      <c r="D82">
+        <v>4330</v>
+      </c>
+      <c r="E82">
+        <f t="shared" si="1"/>
+        <v>8660</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B83" t="s">
+        <v>19</v>
+      </c>
+      <c r="C83">
+        <v>130</v>
+      </c>
+      <c r="D83">
+        <v>4330</v>
+      </c>
+      <c r="E83">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B84" t="s">
+        <v>518</v>
+      </c>
+      <c r="C84">
+        <v>550</v>
+      </c>
+      <c r="D84">
+        <v>4330</v>
+      </c>
+      <c r="E84">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B85" t="s">
+        <v>101</v>
+      </c>
+      <c r="C85">
+        <v>550</v>
+      </c>
+      <c r="D85">
+        <v>4330</v>
+      </c>
+      <c r="E85">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B86" t="s">
+        <v>330</v>
+      </c>
+      <c r="C86">
+        <v>580</v>
+      </c>
+      <c r="D86">
+        <v>4330</v>
+      </c>
+      <c r="E86">
+        <f t="shared" si="1"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B87" t="s">
+        <v>16</v>
+      </c>
+      <c r="C87">
+        <v>130</v>
+      </c>
+      <c r="D87">
+        <v>4330</v>
+      </c>
+      <c r="E87">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B88" t="s">
+        <v>209</v>
+      </c>
+      <c r="C88">
+        <v>408</v>
+      </c>
+      <c r="D88">
+        <v>4330</v>
+      </c>
+      <c r="E88">
+        <f t="shared" si="1"/>
+        <v>1766640</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A89" s="37">
+        <v>46182</v>
+      </c>
+      <c r="B89" t="s">
+        <v>183</v>
+      </c>
+      <c r="C89">
+        <v>550</v>
+      </c>
+      <c r="D89">
+        <v>4330</v>
+      </c>
+      <c r="E89">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B90" t="s">
+        <v>519</v>
+      </c>
+      <c r="C90">
+        <v>550</v>
+      </c>
+      <c r="D90">
+        <v>4330</v>
+      </c>
+      <c r="E90">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B91" t="s">
+        <v>62</v>
+      </c>
+      <c r="C91">
+        <v>550</v>
+      </c>
+      <c r="D91">
+        <v>4330</v>
+      </c>
+      <c r="E91">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B92" t="s">
+        <v>56</v>
+      </c>
+      <c r="C92">
+        <v>550</v>
+      </c>
+      <c r="D92">
+        <v>4330</v>
+      </c>
+      <c r="E92">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B93" t="s">
+        <v>23</v>
+      </c>
+      <c r="C93">
+        <v>550</v>
+      </c>
+      <c r="D93">
+        <v>4330</v>
+      </c>
+      <c r="E93">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B94" t="s">
+        <v>43</v>
+      </c>
+      <c r="C94">
+        <v>550</v>
+      </c>
+      <c r="D94">
+        <v>4330</v>
+      </c>
+      <c r="E94">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B95" t="s">
+        <v>148</v>
+      </c>
+      <c r="C95">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>4330</v>
+      </c>
+      <c r="E95">
+        <f t="shared" si="1"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B96" t="s">
+        <v>95</v>
+      </c>
+      <c r="C96">
+        <v>560</v>
+      </c>
+      <c r="D96">
+        <v>4330</v>
+      </c>
+      <c r="E96">
+        <f t="shared" si="1"/>
+        <v>2424800</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B97" t="s">
+        <v>50</v>
+      </c>
+      <c r="C97">
+        <v>365</v>
+      </c>
+      <c r="D97">
+        <v>4330</v>
+      </c>
+      <c r="E97">
+        <f t="shared" si="1"/>
+        <v>1580450</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
+        <v>40</v>
+      </c>
+      <c r="C98">
+        <v>550</v>
+      </c>
+      <c r="D98">
+        <v>4330</v>
+      </c>
+      <c r="E98">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B99" t="s">
+        <v>3</v>
+      </c>
+      <c r="C99">
+        <v>130</v>
+      </c>
+      <c r="D99">
+        <v>4330</v>
+      </c>
+      <c r="E99">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B100" t="s">
+        <v>394</v>
+      </c>
+      <c r="C100">
+        <v>30</v>
+      </c>
+      <c r="D100">
+        <v>4330</v>
+      </c>
+      <c r="E100">
+        <f t="shared" si="1"/>
+        <v>129900</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B101" t="s">
+        <v>18</v>
+      </c>
+      <c r="C101">
+        <v>325</v>
+      </c>
+      <c r="D101">
+        <v>4330</v>
+      </c>
+      <c r="E101">
+        <f t="shared" si="1"/>
+        <v>1407250</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A102" s="37">
+        <v>46183</v>
+      </c>
+      <c r="B102" t="s">
+        <v>49</v>
+      </c>
+      <c r="C102">
+        <v>548</v>
+      </c>
+      <c r="D102">
+        <v>4330</v>
+      </c>
+      <c r="E102">
+        <f t="shared" si="1"/>
+        <v>2372840</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B103" t="s">
+        <v>520</v>
+      </c>
+      <c r="C103">
+        <v>20</v>
+      </c>
+      <c r="D103">
+        <v>4330</v>
+      </c>
+      <c r="E103">
+        <f t="shared" si="1"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B104" t="s">
+        <v>19</v>
+      </c>
+      <c r="C104">
+        <v>130</v>
+      </c>
+      <c r="D104">
+        <v>4330</v>
+      </c>
+      <c r="E104">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B105" t="s">
+        <v>22</v>
+      </c>
+      <c r="C105">
+        <v>350</v>
+      </c>
+      <c r="D105">
+        <v>4330</v>
+      </c>
+      <c r="E105">
+        <f t="shared" si="1"/>
+        <v>1515500</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B106" t="s">
+        <v>521</v>
+      </c>
+      <c r="C106">
+        <v>20</v>
+      </c>
+      <c r="D106">
+        <v>4330</v>
+      </c>
+      <c r="E106">
+        <f t="shared" si="1"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B107" t="s">
+        <v>25</v>
+      </c>
+      <c r="C107">
+        <v>550</v>
+      </c>
+      <c r="D107">
+        <v>4330</v>
+      </c>
+      <c r="E107">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B108" t="s">
+        <v>378</v>
+      </c>
+      <c r="C108">
+        <v>577</v>
+      </c>
+      <c r="D108">
+        <v>4330</v>
+      </c>
+      <c r="E108">
+        <f t="shared" si="1"/>
+        <v>2498410</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B109" t="s">
+        <v>16</v>
+      </c>
+      <c r="C109">
+        <v>130</v>
+      </c>
+      <c r="D109">
+        <v>4330</v>
+      </c>
+      <c r="E109">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B110" t="s">
+        <v>26</v>
+      </c>
+      <c r="C110">
+        <v>391</v>
+      </c>
+      <c r="D110">
+        <v>4330</v>
+      </c>
+      <c r="E110">
+        <f t="shared" si="1"/>
+        <v>1693030</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A111" s="37">
+        <v>46184</v>
+      </c>
+      <c r="B111" t="s">
+        <v>307</v>
+      </c>
+      <c r="C111">
+        <v>580</v>
+      </c>
+      <c r="D111">
+        <v>4330</v>
+      </c>
+      <c r="E111">
+        <f t="shared" si="1"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B112" t="s">
+        <v>522</v>
+      </c>
+      <c r="C112">
+        <v>550</v>
+      </c>
+      <c r="D112">
+        <v>4330</v>
+      </c>
+      <c r="E112">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B113" t="s">
+        <v>23</v>
+      </c>
+      <c r="C113">
+        <v>550</v>
+      </c>
+      <c r="D113">
+        <v>4330</v>
+      </c>
+      <c r="E113">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B114" t="s">
+        <v>3</v>
+      </c>
+      <c r="C114">
+        <v>130</v>
+      </c>
+      <c r="D114">
+        <v>4330</v>
+      </c>
+      <c r="E114">
+        <f t="shared" si="1"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B115" t="s">
+        <v>50</v>
+      </c>
+      <c r="C115">
+        <v>376</v>
+      </c>
+      <c r="D115">
+        <v>4330</v>
+      </c>
+      <c r="E115">
+        <f t="shared" si="1"/>
+        <v>1628080</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B116" t="s">
+        <v>115</v>
+      </c>
+      <c r="C116">
+        <v>550</v>
+      </c>
+      <c r="D116">
+        <v>4330</v>
+      </c>
+      <c r="E116">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B117" t="s">
+        <v>225</v>
+      </c>
+      <c r="C117">
+        <v>575</v>
+      </c>
+      <c r="D117">
+        <v>4330</v>
+      </c>
+      <c r="E117">
+        <f t="shared" si="1"/>
+        <v>2489750</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B118" t="s">
+        <v>209</v>
+      </c>
+      <c r="C118">
+        <v>402</v>
+      </c>
+      <c r="D118">
+        <v>4330</v>
+      </c>
+      <c r="E118">
+        <f t="shared" si="1"/>
+        <v>1740660</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A119" s="37">
+        <v>46185</v>
+      </c>
+      <c r="B119" t="s">
+        <v>522</v>
+      </c>
+      <c r="C119">
+        <v>2</v>
+      </c>
+      <c r="D119">
+        <v>4330</v>
+      </c>
+      <c r="E119">
+        <f t="shared" si="1"/>
+        <v>8660</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B120" t="s">
+        <v>523</v>
+      </c>
+      <c r="C120">
+        <v>10</v>
+      </c>
+      <c r="D120">
+        <v>4330</v>
+      </c>
+      <c r="E120">
+        <f t="shared" si="1"/>
+        <v>43300</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B121" t="s">
+        <v>210</v>
+      </c>
+      <c r="C121">
+        <v>20</v>
+      </c>
+      <c r="D121">
+        <v>4330</v>
+      </c>
+      <c r="E121">
+        <f t="shared" si="1"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>121</v>
+      </c>
+      <c r="C122">
+        <v>20</v>
+      </c>
+      <c r="D122">
+        <v>4330</v>
+      </c>
+      <c r="E122">
+        <f t="shared" si="1"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B123" t="s">
+        <v>524</v>
+      </c>
+      <c r="C123">
+        <v>570</v>
+      </c>
+      <c r="D123">
+        <v>4330</v>
+      </c>
+      <c r="E123">
+        <f t="shared" si="1"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>525</v>
+      </c>
+      <c r="C124">
+        <v>585</v>
+      </c>
+      <c r="D124">
+        <v>4330</v>
+      </c>
+      <c r="E124">
+        <f t="shared" si="1"/>
+        <v>2533050</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B125" t="s">
+        <v>172</v>
+      </c>
+      <c r="C125">
+        <v>550</v>
+      </c>
+      <c r="D125">
+        <v>4330</v>
+      </c>
+      <c r="E125">
+        <f t="shared" si="1"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B126" t="s">
+        <v>526</v>
+      </c>
+      <c r="C126">
+        <v>590</v>
+      </c>
+      <c r="D126">
+        <v>4330</v>
+      </c>
+      <c r="E126">
+        <f t="shared" si="1"/>
+        <v>2554700</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C127">
+        <v>580</v>
+      </c>
+      <c r="D127">
+        <v>4330</v>
+      </c>
+      <c r="E127">
+        <f t="shared" si="1"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B128" t="s">
+        <v>49</v>
+      </c>
+      <c r="C128">
+        <v>543</v>
+      </c>
+      <c r="D128">
+        <v>4330</v>
+      </c>
+      <c r="E128">
+        <f t="shared" si="1"/>
+        <v>2351190</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B129" t="s">
+        <v>528</v>
+      </c>
+      <c r="C129">
+        <v>20</v>
+      </c>
+      <c r="D129">
+        <v>4330</v>
+      </c>
+      <c r="E129">
+        <f t="shared" ref="E129:E192" si="2">C129*D129</f>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B130" t="s">
+        <v>149</v>
+      </c>
+      <c r="C130">
+        <v>550</v>
+      </c>
+      <c r="D130">
+        <v>4330</v>
+      </c>
+      <c r="E130">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B131" t="s">
+        <v>22</v>
+      </c>
+      <c r="C131">
+        <v>357</v>
+      </c>
+      <c r="D131">
+        <v>4330</v>
+      </c>
+      <c r="E131">
+        <f t="shared" si="2"/>
+        <v>1545810</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B132" t="s">
+        <v>528</v>
+      </c>
+      <c r="C132">
+        <v>577</v>
+      </c>
+      <c r="D132">
+        <v>4330</v>
+      </c>
+      <c r="E132">
+        <f t="shared" si="2"/>
+        <v>2498410</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B133" t="s">
+        <v>529</v>
+      </c>
+      <c r="C133">
+        <v>595</v>
+      </c>
+      <c r="D133">
+        <v>4330</v>
+      </c>
+      <c r="E133">
+        <f t="shared" si="2"/>
+        <v>2576350</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B134" t="s">
+        <v>78</v>
+      </c>
+      <c r="C134">
+        <v>550</v>
+      </c>
+      <c r="D134">
+        <v>4330</v>
+      </c>
+      <c r="E134">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B135" t="s">
+        <v>186</v>
+      </c>
+      <c r="C135">
+        <v>550</v>
+      </c>
+      <c r="D135">
+        <v>4330</v>
+      </c>
+      <c r="E135">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B136" t="s">
+        <v>112</v>
+      </c>
+      <c r="C136">
+        <v>2</v>
+      </c>
+      <c r="D136">
+        <v>4330</v>
+      </c>
+      <c r="E136">
+        <f t="shared" si="2"/>
+        <v>8660</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B137" t="s">
+        <v>16</v>
+      </c>
+      <c r="C137">
+        <v>130</v>
+      </c>
+      <c r="D137">
+        <v>4330</v>
+      </c>
+      <c r="E137">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B138" t="s">
+        <v>521</v>
+      </c>
+      <c r="C138">
+        <v>584</v>
+      </c>
+      <c r="D138">
+        <v>4330</v>
+      </c>
+      <c r="E138">
+        <f t="shared" si="2"/>
+        <v>2528720</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B139" t="s">
+        <v>18</v>
+      </c>
+      <c r="C139">
+        <v>346</v>
+      </c>
+      <c r="D139">
+        <v>4330</v>
+      </c>
+      <c r="E139">
+        <f t="shared" si="2"/>
+        <v>1498180</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B140" t="s">
+        <v>19</v>
+      </c>
+      <c r="C140">
+        <v>130</v>
+      </c>
+      <c r="D140">
+        <v>4330</v>
+      </c>
+      <c r="E140">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A141" s="37">
+        <v>46186</v>
+      </c>
+      <c r="B141" t="s">
+        <v>23</v>
+      </c>
+      <c r="C141">
+        <v>548</v>
+      </c>
+      <c r="D141">
+        <v>4330</v>
+      </c>
+      <c r="E141">
+        <f t="shared" si="2"/>
+        <v>2372840</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B142" t="s">
+        <v>50</v>
+      </c>
+      <c r="C142">
+        <v>363</v>
+      </c>
+      <c r="D142">
+        <v>4330</v>
+      </c>
+      <c r="E142">
+        <f t="shared" si="2"/>
+        <v>1571790</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B143" t="s">
+        <v>394</v>
+      </c>
+      <c r="C143">
+        <v>586</v>
+      </c>
+      <c r="D143">
+        <v>4330</v>
+      </c>
+      <c r="E143">
+        <f t="shared" si="2"/>
+        <v>2537380</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B144" t="s">
+        <v>168</v>
+      </c>
+      <c r="C144">
+        <v>20</v>
+      </c>
+      <c r="D144">
+        <v>4330</v>
+      </c>
+      <c r="E144">
+        <f t="shared" si="2"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B145" t="s">
+        <v>121</v>
+      </c>
+      <c r="C145">
+        <v>580</v>
+      </c>
+      <c r="D145">
+        <v>4330</v>
+      </c>
+      <c r="E145">
+        <f t="shared" si="2"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B146" t="s">
+        <v>3</v>
+      </c>
+      <c r="C146">
+        <v>130</v>
+      </c>
+      <c r="D146">
+        <v>4330</v>
+      </c>
+      <c r="E146">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B147" t="s">
+        <v>26</v>
+      </c>
+      <c r="C147">
+        <v>399</v>
+      </c>
+      <c r="D147">
+        <v>4330</v>
+      </c>
+      <c r="E147">
+        <f t="shared" si="2"/>
+        <v>1727670</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B148" t="s">
+        <v>49</v>
+      </c>
+      <c r="C148">
+        <v>550</v>
+      </c>
+      <c r="D148">
+        <v>4330</v>
+      </c>
+      <c r="E148">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B149" t="s">
+        <v>22</v>
+      </c>
+      <c r="C149">
+        <v>347</v>
+      </c>
+      <c r="D149">
+        <v>4330</v>
+      </c>
+      <c r="E149">
+        <f t="shared" si="2"/>
+        <v>1502510</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B150" t="s">
+        <v>16</v>
+      </c>
+      <c r="C150">
+        <v>130</v>
+      </c>
+      <c r="D150">
+        <v>4330</v>
+      </c>
+      <c r="E150">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B151" t="s">
+        <v>209</v>
+      </c>
+      <c r="C151">
+        <v>380</v>
+      </c>
+      <c r="D151">
+        <v>4330</v>
+      </c>
+      <c r="E151">
+        <f t="shared" si="2"/>
+        <v>1645400</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B152" t="s">
+        <v>19</v>
+      </c>
+      <c r="C152">
+        <v>130</v>
+      </c>
+      <c r="D152">
+        <v>4330</v>
+      </c>
+      <c r="E152">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A153" s="37">
+        <v>46187</v>
+      </c>
+      <c r="B153" t="s">
+        <v>239</v>
+      </c>
+      <c r="C153">
+        <v>560</v>
+      </c>
+      <c r="D153">
+        <v>4330</v>
+      </c>
+      <c r="E153">
+        <f t="shared" si="2"/>
+        <v>2424800</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B154" t="s">
+        <v>23</v>
+      </c>
+      <c r="C154">
+        <v>550</v>
+      </c>
+      <c r="D154">
+        <v>4330</v>
+      </c>
+      <c r="E154">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B155" t="s">
+        <v>530</v>
+      </c>
+      <c r="C155">
+        <v>520</v>
+      </c>
+      <c r="D155">
+        <v>4330</v>
+      </c>
+      <c r="E155">
+        <f t="shared" si="2"/>
+        <v>2251600</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B156" t="s">
+        <v>50</v>
+      </c>
+      <c r="C156">
+        <v>333</v>
+      </c>
+      <c r="D156">
+        <v>4330</v>
+      </c>
+      <c r="E156">
+        <f t="shared" si="2"/>
+        <v>1441890</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B157" t="s">
+        <v>531</v>
+      </c>
+      <c r="C157">
+        <v>565</v>
+      </c>
+      <c r="D157">
+        <v>4330</v>
+      </c>
+      <c r="E157">
+        <f t="shared" si="2"/>
+        <v>2446450</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B158" t="s">
+        <v>243</v>
+      </c>
+      <c r="C158">
+        <v>550</v>
+      </c>
+      <c r="D158">
+        <v>4330</v>
+      </c>
+      <c r="E158">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B159" t="s">
+        <v>396</v>
+      </c>
+      <c r="C159">
+        <v>550</v>
+      </c>
+      <c r="D159">
+        <v>4330</v>
+      </c>
+      <c r="E159">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B160" t="s">
+        <v>128</v>
+      </c>
+      <c r="C160">
+        <v>550</v>
+      </c>
+      <c r="D160">
+        <v>4330</v>
+      </c>
+      <c r="E160">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B161" t="s">
+        <v>112</v>
+      </c>
+      <c r="C161">
+        <v>550</v>
+      </c>
+      <c r="D161">
+        <v>4330</v>
+      </c>
+      <c r="E161">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A162" s="37">
+        <v>46190</v>
+      </c>
+      <c r="B162" t="s">
+        <v>122</v>
+      </c>
+      <c r="C162">
+        <v>20</v>
+      </c>
+      <c r="D162">
+        <v>4330</v>
+      </c>
+      <c r="E162">
+        <f t="shared" si="2"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B163" t="s">
+        <v>23</v>
+      </c>
+      <c r="C163">
+        <v>550</v>
+      </c>
+      <c r="D163">
+        <v>4330</v>
+      </c>
+      <c r="E163">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B164" t="s">
+        <v>148</v>
+      </c>
+      <c r="C164">
+        <v>465</v>
+      </c>
+      <c r="D164">
+        <v>4330</v>
+      </c>
+      <c r="E164">
+        <f t="shared" si="2"/>
+        <v>2013450</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B165" t="s">
+        <v>299</v>
+      </c>
+      <c r="C165">
+        <v>80</v>
+      </c>
+      <c r="D165">
+        <v>4330</v>
+      </c>
+      <c r="E165">
+        <f t="shared" si="2"/>
+        <v>346400</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B166" t="s">
+        <v>22</v>
+      </c>
+      <c r="C166">
+        <v>352</v>
+      </c>
+      <c r="D166">
+        <v>4330</v>
+      </c>
+      <c r="E166">
+        <f t="shared" si="2"/>
+        <v>1524160</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B167" t="s">
+        <v>45</v>
+      </c>
+      <c r="C167">
+        <v>550</v>
+      </c>
+      <c r="D167">
+        <v>4330</v>
+      </c>
+      <c r="E167">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B168" t="s">
+        <v>257</v>
+      </c>
+      <c r="C168">
+        <v>550</v>
+      </c>
+      <c r="D168">
+        <v>4330</v>
+      </c>
+      <c r="E168">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B169" t="s">
+        <v>109</v>
+      </c>
+      <c r="C169">
+        <v>550</v>
+      </c>
+      <c r="D169">
+        <v>4330</v>
+      </c>
+      <c r="E169">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B170" t="s">
+        <v>234</v>
+      </c>
+      <c r="C170">
+        <v>437</v>
+      </c>
+      <c r="D170">
+        <v>4330</v>
+      </c>
+      <c r="E170">
+        <f t="shared" si="2"/>
+        <v>1892210</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B171" t="s">
+        <v>123</v>
+      </c>
+      <c r="C171">
+        <v>550</v>
+      </c>
+      <c r="D171">
+        <v>4330</v>
+      </c>
+      <c r="E171">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B172" t="s">
+        <v>133</v>
+      </c>
+      <c r="C172">
+        <v>550</v>
+      </c>
+      <c r="D172">
+        <v>4330</v>
+      </c>
+      <c r="E172">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B173" t="s">
+        <v>50</v>
+      </c>
+      <c r="C173">
+        <v>365</v>
+      </c>
+      <c r="D173">
+        <v>4330</v>
+      </c>
+      <c r="E173">
+        <f t="shared" si="2"/>
+        <v>1580450</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B174" t="s">
+        <v>3</v>
+      </c>
+      <c r="C174">
+        <v>130</v>
+      </c>
+      <c r="D174">
+        <v>4330</v>
+      </c>
+      <c r="E174">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B175" t="s">
+        <v>209</v>
+      </c>
+      <c r="C175">
+        <v>369</v>
+      </c>
+      <c r="D175">
+        <v>4330</v>
+      </c>
+      <c r="E175">
+        <f t="shared" si="2"/>
+        <v>1597770</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A176" s="37">
+        <v>46191</v>
+      </c>
+      <c r="B176" t="s">
+        <v>19</v>
+      </c>
+      <c r="C176">
+        <v>130</v>
+      </c>
+      <c r="D176">
+        <v>4330</v>
+      </c>
+      <c r="E176">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B177" t="s">
+        <v>194</v>
+      </c>
+      <c r="C177">
+        <v>550</v>
+      </c>
+      <c r="D177">
+        <v>4330</v>
+      </c>
+      <c r="E177">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B178" t="s">
+        <v>122</v>
+      </c>
+      <c r="C178">
+        <v>570</v>
+      </c>
+      <c r="D178">
+        <v>4330</v>
+      </c>
+      <c r="E178">
+        <f t="shared" si="2"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B179" t="s">
+        <v>49</v>
+      </c>
+      <c r="C179">
+        <v>535</v>
+      </c>
+      <c r="D179">
+        <v>4330</v>
+      </c>
+      <c r="E179">
+        <f t="shared" si="2"/>
+        <v>2316550</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B180" t="s">
+        <v>532</v>
+      </c>
+      <c r="C180">
+        <v>550</v>
+      </c>
+      <c r="D180">
+        <v>4330</v>
+      </c>
+      <c r="E180">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B181" t="s">
+        <v>242</v>
+      </c>
+      <c r="C181">
+        <v>550</v>
+      </c>
+      <c r="D181">
+        <v>4330</v>
+      </c>
+      <c r="E181">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B182" t="s">
+        <v>174</v>
+      </c>
+      <c r="C182">
+        <v>550</v>
+      </c>
+      <c r="D182">
+        <v>4330</v>
+      </c>
+      <c r="E182">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B183" t="s">
+        <v>4</v>
+      </c>
+      <c r="C183">
+        <v>343</v>
+      </c>
+      <c r="D183">
+        <v>4330</v>
+      </c>
+      <c r="E183">
+        <f t="shared" si="2"/>
+        <v>1485190</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B184" t="s">
+        <v>392</v>
+      </c>
+      <c r="C184">
+        <v>550</v>
+      </c>
+      <c r="D184">
+        <v>4330</v>
+      </c>
+      <c r="E184">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B185" t="s">
+        <v>533</v>
+      </c>
+      <c r="C185">
+        <v>555</v>
+      </c>
+      <c r="D185">
+        <v>4330</v>
+      </c>
+      <c r="E185">
+        <f t="shared" si="2"/>
+        <v>2403150</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B186" t="s">
+        <v>416</v>
+      </c>
+      <c r="C186">
+        <v>20</v>
+      </c>
+      <c r="D186">
+        <v>4330</v>
+      </c>
+      <c r="E186">
+        <f t="shared" si="2"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B187" t="s">
+        <v>534</v>
+      </c>
+      <c r="C187">
+        <v>556</v>
+      </c>
+      <c r="D187">
+        <v>4330</v>
+      </c>
+      <c r="E187">
+        <f t="shared" si="2"/>
+        <v>2407480</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B188" t="s">
+        <v>386</v>
+      </c>
+      <c r="C188">
+        <v>550</v>
+      </c>
+      <c r="D188">
+        <v>4330</v>
+      </c>
+      <c r="E188">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B189" t="s">
+        <v>329</v>
+      </c>
+      <c r="C189">
+        <v>550</v>
+      </c>
+      <c r="D189">
+        <v>4330</v>
+      </c>
+      <c r="E189">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B190" t="s">
+        <v>16</v>
+      </c>
+      <c r="C190">
+        <v>130</v>
+      </c>
+      <c r="D190">
+        <v>4330</v>
+      </c>
+      <c r="E190">
+        <f t="shared" si="2"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B191" t="s">
+        <v>535</v>
+      </c>
+      <c r="C191">
+        <v>334</v>
+      </c>
+      <c r="D191">
+        <v>4330</v>
+      </c>
+      <c r="E191">
+        <f t="shared" si="2"/>
+        <v>1446220</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A192" s="37">
+        <v>46192</v>
+      </c>
+      <c r="B192" t="s">
+        <v>23</v>
+      </c>
+      <c r="C192">
+        <v>550</v>
+      </c>
+      <c r="D192">
+        <v>4330</v>
+      </c>
+      <c r="E192">
+        <f t="shared" si="2"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B193" t="s">
+        <v>127</v>
+      </c>
+      <c r="C193">
+        <v>550</v>
+      </c>
+      <c r="D193">
+        <v>4330</v>
+      </c>
+      <c r="E193">
+        <f t="shared" ref="E193:E216" si="3">C193*D193</f>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B194" t="s">
+        <v>151</v>
+      </c>
+      <c r="C194">
+        <v>550</v>
+      </c>
+      <c r="D194">
+        <v>4330</v>
+      </c>
+      <c r="E194">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B195" t="s">
+        <v>22</v>
+      </c>
+      <c r="C195">
+        <v>352</v>
+      </c>
+      <c r="D195">
+        <v>4330</v>
+      </c>
+      <c r="E195">
+        <f t="shared" si="3"/>
+        <v>1524160</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B196" t="s">
+        <v>536</v>
+      </c>
+      <c r="C196">
+        <v>20</v>
+      </c>
+      <c r="D196">
+        <v>4330</v>
+      </c>
+      <c r="E196">
+        <f t="shared" si="3"/>
+        <v>86600</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B197" t="s">
+        <v>287</v>
+      </c>
+      <c r="C197">
+        <v>586</v>
+      </c>
+      <c r="D197">
+        <v>4330</v>
+      </c>
+      <c r="E197">
+        <f t="shared" si="3"/>
+        <v>2537380</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B198" t="s">
+        <v>204</v>
+      </c>
+      <c r="C198">
+        <v>550</v>
+      </c>
+      <c r="D198">
+        <v>4330</v>
+      </c>
+      <c r="E198">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B199" t="s">
+        <v>80</v>
+      </c>
+      <c r="C199">
+        <v>550</v>
+      </c>
+      <c r="D199">
+        <v>4330</v>
+      </c>
+      <c r="E199">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B200" t="s">
+        <v>3</v>
+      </c>
+      <c r="C200">
+        <v>130</v>
+      </c>
+      <c r="D200">
+        <v>4330</v>
+      </c>
+      <c r="E200">
+        <f t="shared" si="3"/>
+        <v>562900</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B201" t="s">
+        <v>26</v>
+      </c>
+      <c r="C201">
+        <v>373</v>
+      </c>
+      <c r="D201">
+        <v>4330</v>
+      </c>
+      <c r="E201">
+        <f t="shared" si="3"/>
+        <v>1615090</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A202" s="37">
+        <v>46193</v>
+      </c>
+      <c r="B202" t="s">
+        <v>15</v>
+      </c>
+      <c r="C202">
+        <v>2</v>
+      </c>
+      <c r="D202">
+        <v>4330</v>
+      </c>
+      <c r="E202">
+        <f t="shared" si="3"/>
+        <v>8660</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B203" t="s">
+        <v>24</v>
+      </c>
+      <c r="C203">
+        <v>2</v>
+      </c>
+      <c r="D203">
+        <v>4330</v>
+      </c>
+      <c r="E203">
+        <f t="shared" si="3"/>
+        <v>8660</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B204" t="s">
+        <v>537</v>
+      </c>
+      <c r="C204">
+        <v>555</v>
+      </c>
+      <c r="D204">
+        <v>4330</v>
+      </c>
+      <c r="E204">
+        <f t="shared" si="3"/>
+        <v>2403150</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B205" t="s">
+        <v>126</v>
+      </c>
+      <c r="C205">
+        <v>575</v>
+      </c>
+      <c r="D205">
+        <v>4330</v>
+      </c>
+      <c r="E205">
+        <f t="shared" si="3"/>
+        <v>2489750</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B206" t="s">
+        <v>49</v>
+      </c>
+      <c r="C206">
+        <v>546</v>
+      </c>
+      <c r="D206">
+        <v>4330</v>
+      </c>
+      <c r="E206">
+        <f t="shared" si="3"/>
+        <v>2364180</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B207" t="s">
+        <v>159</v>
+      </c>
+      <c r="C207">
+        <v>565</v>
+      </c>
+      <c r="D207">
+        <v>4330</v>
+      </c>
+      <c r="E207">
+        <f t="shared" si="3"/>
+        <v>2446450</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B208" t="s">
+        <v>131</v>
+      </c>
+      <c r="C208">
+        <v>550</v>
+      </c>
+      <c r="D208">
+        <v>4330</v>
+      </c>
+      <c r="E208">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B209" t="s">
+        <v>351</v>
+      </c>
+      <c r="C209">
+        <v>570</v>
+      </c>
+      <c r="D209">
+        <v>4330</v>
+      </c>
+      <c r="E209">
+        <f t="shared" si="3"/>
+        <v>2468100</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B210" t="s">
+        <v>154</v>
+      </c>
+      <c r="C210">
+        <v>550</v>
+      </c>
+      <c r="D210">
+        <v>4330</v>
+      </c>
+      <c r="E210">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B211" t="s">
+        <v>209</v>
+      </c>
+      <c r="C211">
+        <v>363</v>
+      </c>
+      <c r="D211">
+        <v>4330</v>
+      </c>
+      <c r="E211">
+        <f t="shared" si="3"/>
+        <v>1571790</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B212" t="s">
+        <v>23</v>
+      </c>
+      <c r="C212">
+        <v>550</v>
+      </c>
+      <c r="D212">
+        <v>4330</v>
+      </c>
+      <c r="E212">
+        <f t="shared" si="3"/>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B213" t="s">
+        <v>4</v>
+      </c>
+      <c r="C213">
+        <v>346</v>
+      </c>
+      <c r="D213">
+        <v>4330</v>
+      </c>
+      <c r="E213">
+        <f t="shared" si="3"/>
+        <v>1498180</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A214" s="37">
+        <v>46195</v>
+      </c>
+      <c r="B214" t="s">
+        <v>145</v>
+      </c>
+      <c r="C214">
+        <v>580</v>
+      </c>
+      <c r="D214">
+        <v>4330</v>
+      </c>
+      <c r="E214">
+        <f t="shared" si="3"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B215" t="s">
+        <v>416</v>
+      </c>
+      <c r="C215">
+        <v>580</v>
+      </c>
+      <c r="D215">
+        <v>4330</v>
+      </c>
+      <c r="E215">
+        <f t="shared" si="3"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B216" t="s">
+        <v>108</v>
+      </c>
+      <c r="C216">
+        <v>546</v>
+      </c>
+      <c r="D216">
+        <v>4330</v>
+      </c>
+      <c r="E216">
+        <f t="shared" si="3"/>
+        <v>2364180</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed issues with lpo format
</commit_message>
<xml_diff>
--- a/dar yard lpos.xlsx
+++ b/dar yard lpos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tungsten\Documents\Backup from old pc\WINDOWS 11\Fuel_Order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5297E8AE-EC1C-4A2B-8686-1BB0BD8B0A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DBA497-7EE5-40CB-807A-32347F3A68CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="5" xr2:uid="{644A8DE3-68DC-4C6A-A18C-611A87002412}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{644A8DE3-68DC-4C6A-A18C-611A87002412}"/>
   </bookViews>
   <sheets>
     <sheet name="JAN" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1404" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="538">
   <si>
     <t>DATE</t>
   </si>
@@ -20616,33 +20616,35 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C60458-4749-4ACB-9FC1-AAB0CFF01868}">
-  <dimension ref="A1:E216"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="37">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="37">
         <v>46174</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>499</v>
-      </c>
-      <c r="C1">
-        <v>550</v>
-      </c>
-      <c r="D1">
-        <v>4330</v>
-      </c>
-      <c r="E1">
-        <f t="shared" ref="E1:E64" si="0">C1*D1</f>
-        <v>2381500</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>374</v>
       </c>
       <c r="C2">
         <v>550</v>
@@ -20651,43 +20653,43 @@
         <v>4330</v>
       </c>
       <c r="E2">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E2:E65" si="0">C2*D2</f>
         <v>2381500</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>394</v>
+        <v>374</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>550</v>
       </c>
       <c r="D3">
         <v>4330</v>
       </c>
       <c r="E3">
         <f t="shared" si="0"/>
-        <v>21650</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>500</v>
+        <v>394</v>
       </c>
       <c r="C4">
-        <v>550</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>4330</v>
       </c>
       <c r="E4">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>21650</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>137</v>
+        <v>500</v>
       </c>
       <c r="C5">
         <v>550</v>
@@ -20702,7 +20704,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C6">
         <v>550</v>
@@ -20717,7 +20719,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>501</v>
+        <v>132</v>
       </c>
       <c r="C7">
         <v>550</v>
@@ -20732,7 +20734,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C8">
         <v>550</v>
@@ -20747,52 +20749,52 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>23</v>
+        <v>502</v>
       </c>
       <c r="C9">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="D9">
         <v>4330</v>
       </c>
       <c r="E9">
         <f t="shared" si="0"/>
-        <v>2299230</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>503</v>
+        <v>23</v>
       </c>
       <c r="C10">
-        <v>573</v>
+        <v>531</v>
       </c>
       <c r="D10">
         <v>4330</v>
       </c>
       <c r="E10">
         <f t="shared" si="0"/>
-        <v>2481090</v>
+        <v>2299230</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C11">
-        <v>550</v>
+        <v>573</v>
       </c>
       <c r="D11">
         <v>4330</v>
       </c>
       <c r="E11">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>2481090</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>323</v>
+        <v>504</v>
       </c>
       <c r="C12">
         <v>550</v>
@@ -20807,7 +20809,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>93</v>
+        <v>323</v>
       </c>
       <c r="C13">
         <v>550</v>
@@ -20822,7 +20824,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>505</v>
+        <v>93</v>
       </c>
       <c r="C14">
         <v>550</v>
@@ -20837,7 +20839,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>334</v>
+        <v>505</v>
       </c>
       <c r="C15">
         <v>550</v>
@@ -20852,37 +20854,37 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>22</v>
+        <v>334</v>
       </c>
       <c r="C16">
-        <v>345</v>
+        <v>550</v>
       </c>
       <c r="D16">
         <v>4330</v>
       </c>
       <c r="E16">
         <f t="shared" si="0"/>
-        <v>1493850</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>293</v>
+        <v>22</v>
       </c>
       <c r="C17">
-        <v>550</v>
+        <v>345</v>
       </c>
       <c r="D17">
         <v>4330</v>
       </c>
       <c r="E17">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>1493850</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>380</v>
+        <v>293</v>
       </c>
       <c r="C18">
         <v>550</v>
@@ -20897,37 +20899,37 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>506</v>
+        <v>380</v>
       </c>
       <c r="C19">
-        <v>517</v>
+        <v>550</v>
       </c>
       <c r="D19">
         <v>4330</v>
       </c>
       <c r="E19">
         <f t="shared" si="0"/>
-        <v>2238610</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
-        <v>3</v>
+        <v>506</v>
       </c>
       <c r="C20">
-        <v>130</v>
+        <v>517</v>
       </c>
       <c r="D20">
         <v>4330</v>
       </c>
       <c r="E20">
         <f t="shared" si="0"/>
-        <v>562900</v>
+        <v>2238610</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C21">
         <v>130</v>
@@ -20941,467 +20943,467 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="37">
-        <v>46175</v>
-      </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C22">
-        <v>370</v>
+        <v>130</v>
       </c>
       <c r="D22">
         <v>4330</v>
       </c>
       <c r="E22">
         <f t="shared" si="0"/>
-        <v>1602100</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="37">
+        <v>46175</v>
+      </c>
       <c r="B23" t="s">
-        <v>371</v>
+        <v>26</v>
       </c>
       <c r="C23">
-        <v>570</v>
+        <v>370</v>
       </c>
       <c r="D23">
         <v>4330</v>
       </c>
       <c r="E23">
         <f t="shared" si="0"/>
-        <v>2468100</v>
+        <v>1602100</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
-        <v>49</v>
+        <v>371</v>
       </c>
       <c r="C24">
-        <v>523</v>
+        <v>570</v>
       </c>
       <c r="D24">
         <v>4330</v>
       </c>
       <c r="E24">
         <f t="shared" si="0"/>
-        <v>2264590</v>
+        <v>2468100</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
-        <v>507</v>
+        <v>49</v>
       </c>
       <c r="C25">
-        <v>590</v>
+        <v>523</v>
       </c>
       <c r="D25">
         <v>4330</v>
       </c>
       <c r="E25">
         <f t="shared" si="0"/>
-        <v>2554700</v>
+        <v>2264590</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
-        <v>50</v>
+        <v>507</v>
       </c>
       <c r="C26">
-        <v>370</v>
+        <v>590</v>
       </c>
       <c r="D26">
         <v>4330</v>
       </c>
       <c r="E26">
         <f t="shared" si="0"/>
-        <v>1602100</v>
+        <v>2554700</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>508</v>
+        <v>50</v>
       </c>
       <c r="C27">
-        <v>5</v>
+        <v>370</v>
       </c>
       <c r="D27">
         <v>4330</v>
       </c>
       <c r="E27">
         <f t="shared" si="0"/>
-        <v>21650</v>
+        <v>1602100</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
-        <v>4</v>
+        <v>508</v>
       </c>
       <c r="C28">
-        <v>338</v>
+        <v>5</v>
       </c>
       <c r="D28">
         <v>4330</v>
       </c>
       <c r="E28">
         <f t="shared" si="0"/>
-        <v>1463540</v>
+        <v>21650</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
-        <v>509</v>
+        <v>4</v>
       </c>
       <c r="C29">
-        <v>550</v>
+        <v>338</v>
       </c>
       <c r="D29">
         <v>4330</v>
       </c>
       <c r="E29">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>1463540</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
-        <v>251</v>
+        <v>509</v>
       </c>
       <c r="C30">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="D30">
         <v>4330</v>
       </c>
       <c r="E30">
         <f t="shared" si="0"/>
-        <v>2338200</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
-        <v>19</v>
+        <v>251</v>
       </c>
       <c r="C31">
-        <v>130</v>
+        <v>540</v>
       </c>
       <c r="D31">
         <v>4330</v>
       </c>
       <c r="E31">
         <f t="shared" si="0"/>
-        <v>562900</v>
+        <v>2338200</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="C32">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="D32">
         <v>4330</v>
       </c>
       <c r="E32">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="37">
-        <v>46176</v>
-      </c>
       <c r="B33" t="s">
-        <v>209</v>
+        <v>97</v>
       </c>
       <c r="C33">
-        <v>370</v>
+        <v>550</v>
       </c>
       <c r="D33">
         <v>4330</v>
       </c>
       <c r="E33">
         <f t="shared" si="0"/>
-        <v>1602100</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="37">
+        <v>46176</v>
+      </c>
       <c r="B34" t="s">
-        <v>23</v>
+        <v>209</v>
       </c>
       <c r="C34">
-        <v>550</v>
+        <v>370</v>
       </c>
       <c r="D34">
         <v>4330</v>
       </c>
       <c r="E34">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>1602100</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C35">
-        <v>350</v>
+        <v>550</v>
       </c>
       <c r="D35">
         <v>4330</v>
       </c>
       <c r="E35">
         <f t="shared" si="0"/>
-        <v>1515500</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
-        <v>451</v>
+        <v>22</v>
       </c>
       <c r="C36">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="D36">
         <v>4330</v>
       </c>
       <c r="E36">
         <f t="shared" si="0"/>
-        <v>519600</v>
+        <v>1515500</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
-        <v>3</v>
+        <v>451</v>
       </c>
       <c r="C37">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D37">
         <v>4330</v>
       </c>
       <c r="E37">
         <f t="shared" si="0"/>
-        <v>562900</v>
+        <v>519600</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
-        <v>328</v>
+        <v>3</v>
       </c>
       <c r="C38">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="D38">
         <v>4330</v>
       </c>
       <c r="E38">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
-        <v>57</v>
+        <v>328</v>
       </c>
       <c r="C39">
-        <v>580</v>
+        <v>550</v>
       </c>
       <c r="D39">
         <v>4330</v>
       </c>
       <c r="E39">
         <f t="shared" si="0"/>
-        <v>2511400</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="37">
-        <v>46177</v>
-      </c>
       <c r="B40" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="C40">
-        <v>334</v>
+        <v>580</v>
       </c>
       <c r="D40">
         <v>4330</v>
       </c>
       <c r="E40">
         <f t="shared" si="0"/>
-        <v>1446220</v>
+        <v>2511400</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="37">
+        <v>46177</v>
+      </c>
       <c r="B41" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="C41">
-        <v>533</v>
+        <v>334</v>
       </c>
       <c r="D41">
         <v>4330</v>
       </c>
       <c r="E41">
         <f t="shared" si="0"/>
-        <v>2307890</v>
+        <v>1446220</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
-        <v>510</v>
+        <v>49</v>
       </c>
       <c r="C42">
-        <v>458</v>
+        <v>533</v>
       </c>
       <c r="D42">
         <v>4330</v>
       </c>
       <c r="E42">
         <f t="shared" si="0"/>
-        <v>1983140</v>
+        <v>2307890</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
-        <v>121</v>
+        <v>510</v>
       </c>
       <c r="C43">
-        <v>20</v>
+        <v>458</v>
       </c>
       <c r="D43">
         <v>4330</v>
       </c>
       <c r="E43">
         <f t="shared" si="0"/>
-        <v>86600</v>
+        <v>1983140</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="C44">
-        <v>550</v>
+        <v>20</v>
       </c>
       <c r="D44">
         <v>4330</v>
       </c>
       <c r="E44">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="C45">
-        <v>5</v>
+        <v>550</v>
       </c>
       <c r="D45">
         <v>4330</v>
       </c>
       <c r="E45">
         <f t="shared" si="0"/>
-        <v>21650</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C46">
-        <v>550</v>
+        <v>5</v>
       </c>
       <c r="D46">
         <v>4330</v>
       </c>
       <c r="E46">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>21650</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
-        <v>511</v>
+        <v>38</v>
       </c>
       <c r="C47">
-        <v>575</v>
+        <v>550</v>
       </c>
       <c r="D47">
         <v>4330</v>
       </c>
       <c r="E47">
         <f t="shared" si="0"/>
-        <v>2489750</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
-        <v>91</v>
+        <v>511</v>
       </c>
       <c r="C48">
-        <v>550</v>
+        <v>575</v>
       </c>
       <c r="D48">
         <v>4330</v>
       </c>
       <c r="E48">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>2489750</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="C49">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D49">
         <v>4330</v>
       </c>
       <c r="E49">
         <f t="shared" si="0"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C50">
-        <v>20</v>
+        <v>130</v>
       </c>
       <c r="D50">
         <v>4330</v>
       </c>
       <c r="E50">
         <f t="shared" si="0"/>
-        <v>86600</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="C51">
-        <v>550</v>
+        <v>20</v>
       </c>
       <c r="D51">
         <v>4330</v>
       </c>
       <c r="E51">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
-        <v>512</v>
+        <v>117</v>
       </c>
       <c r="C52">
         <v>550</v>
@@ -21416,22 +21418,22 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
-        <v>19</v>
+        <v>512</v>
       </c>
       <c r="C53">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D53">
         <v>4330</v>
       </c>
       <c r="E53">
         <f t="shared" si="0"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C54">
         <v>130</v>
@@ -21445,26 +21447,26 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="37">
-        <v>46178</v>
-      </c>
       <c r="B55" t="s">
-        <v>513</v>
+        <v>3</v>
       </c>
       <c r="C55">
-        <v>570</v>
+        <v>130</v>
       </c>
       <c r="D55">
         <v>4330</v>
       </c>
       <c r="E55">
         <f t="shared" si="0"/>
-        <v>2468100</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="37">
+        <v>46178</v>
+      </c>
       <c r="B56" t="s">
-        <v>33</v>
+        <v>513</v>
       </c>
       <c r="C56">
         <v>570</v>
@@ -21479,433 +21481,433 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
-        <v>514</v>
+        <v>33</v>
       </c>
       <c r="C57">
-        <v>597</v>
+        <v>570</v>
       </c>
       <c r="D57">
         <v>4330</v>
       </c>
       <c r="E57">
         <f t="shared" si="0"/>
-        <v>2585010</v>
+        <v>2468100</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
-        <v>23</v>
+        <v>514</v>
       </c>
       <c r="C58">
-        <v>550</v>
+        <v>597</v>
       </c>
       <c r="D58">
         <v>4330</v>
       </c>
       <c r="E58">
         <f t="shared" si="0"/>
-        <v>2381500</v>
+        <v>2585010</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="C59">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="D59">
         <v>4330</v>
       </c>
       <c r="E59">
         <f t="shared" si="0"/>
-        <v>2251600</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
-        <v>515</v>
+        <v>94</v>
       </c>
       <c r="C60">
-        <v>20</v>
+        <v>520</v>
       </c>
       <c r="D60">
         <v>4330</v>
       </c>
       <c r="E60">
         <f t="shared" si="0"/>
-        <v>86600</v>
+        <v>2251600</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
-        <v>4</v>
+        <v>515</v>
       </c>
       <c r="C61">
-        <v>362</v>
+        <v>20</v>
       </c>
       <c r="D61">
         <v>4330</v>
       </c>
       <c r="E61">
         <f t="shared" si="0"/>
-        <v>1567460</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="C62">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="D62">
         <v>4330</v>
       </c>
       <c r="E62">
         <f t="shared" si="0"/>
-        <v>1537150</v>
+        <v>1567460</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="C63">
-        <v>524</v>
+        <v>355</v>
       </c>
       <c r="D63">
         <v>4330</v>
       </c>
       <c r="E63">
         <f t="shared" si="0"/>
-        <v>2268920</v>
+        <v>1537150</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="C64">
-        <v>394</v>
+        <v>524</v>
       </c>
       <c r="D64">
         <v>4330</v>
       </c>
       <c r="E64">
         <f t="shared" si="0"/>
-        <v>1706020</v>
+        <v>2268920</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="37">
-        <v>46179</v>
-      </c>
       <c r="B65" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="C65">
-        <v>541</v>
+        <v>394</v>
       </c>
       <c r="D65">
         <v>4330</v>
       </c>
       <c r="E65">
-        <f t="shared" ref="E65:E128" si="1">C65*D65</f>
-        <v>2342530</v>
+        <f t="shared" si="0"/>
+        <v>1706020</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" s="37">
+        <v>46179</v>
+      </c>
       <c r="B66" t="s">
-        <v>516</v>
+        <v>49</v>
       </c>
       <c r="C66">
-        <v>575</v>
+        <v>541</v>
       </c>
       <c r="D66">
         <v>4330</v>
       </c>
       <c r="E66">
-        <f t="shared" si="1"/>
-        <v>2489750</v>
+        <f t="shared" ref="E66:E129" si="1">C66*D66</f>
+        <v>2342530</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
-        <v>189</v>
+        <v>516</v>
       </c>
       <c r="C67">
-        <v>90</v>
+        <v>575</v>
       </c>
       <c r="D67">
         <v>4330</v>
       </c>
       <c r="E67">
         <f t="shared" si="1"/>
-        <v>389700</v>
+        <v>2489750</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
-        <v>508</v>
+        <v>189</v>
       </c>
       <c r="C68">
-        <v>592</v>
+        <v>90</v>
       </c>
       <c r="D68">
         <v>4330</v>
       </c>
       <c r="E68">
         <f t="shared" si="1"/>
-        <v>2563360</v>
+        <v>389700</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
-        <v>89</v>
+        <v>508</v>
       </c>
       <c r="C69">
-        <v>550</v>
+        <v>592</v>
       </c>
       <c r="D69">
         <v>4330</v>
       </c>
       <c r="E69">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>2563360</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="C70">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D70">
         <v>4330</v>
       </c>
       <c r="E70">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
-        <v>140</v>
+        <v>19</v>
       </c>
       <c r="C71">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="D71">
         <v>4330</v>
       </c>
       <c r="E71">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="C72">
-        <v>370</v>
+        <v>550</v>
       </c>
       <c r="D72">
         <v>4330</v>
       </c>
       <c r="E72">
         <f t="shared" si="1"/>
-        <v>1602100</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="C73">
-        <v>130</v>
+        <v>370</v>
       </c>
       <c r="D73">
         <v>4330</v>
       </c>
       <c r="E73">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>1602100</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
-        <v>209</v>
+        <v>16</v>
       </c>
       <c r="C74">
-        <v>406</v>
+        <v>130</v>
       </c>
       <c r="D74">
         <v>4330</v>
       </c>
       <c r="E74">
         <f t="shared" si="1"/>
-        <v>1757980</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
-        <v>18</v>
+        <v>209</v>
       </c>
       <c r="C75">
-        <v>348</v>
+        <v>406</v>
       </c>
       <c r="D75">
         <v>4330</v>
       </c>
       <c r="E75">
         <f t="shared" si="1"/>
-        <v>1506840</v>
+        <v>1757980</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C76">
-        <v>550</v>
+        <v>348</v>
       </c>
       <c r="D76">
         <v>4330</v>
       </c>
       <c r="E76">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>1506840</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C77">
-        <v>352</v>
+        <v>550</v>
       </c>
       <c r="D77">
         <v>4330</v>
       </c>
       <c r="E77">
         <f t="shared" si="1"/>
-        <v>1524160</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C78">
-        <v>130</v>
+        <v>352</v>
       </c>
       <c r="D78">
         <v>4330</v>
       </c>
       <c r="E78">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>1524160</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="C79">
-        <v>386</v>
+        <v>130</v>
       </c>
       <c r="D79">
         <v>4330</v>
       </c>
       <c r="E79">
         <f t="shared" si="1"/>
-        <v>1671380</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" s="37">
-        <v>46181</v>
-      </c>
       <c r="B80" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="C80">
-        <v>536</v>
+        <v>386</v>
       </c>
       <c r="D80">
         <v>4330</v>
       </c>
       <c r="E80">
         <f t="shared" si="1"/>
-        <v>2320880</v>
+        <v>1671380</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" s="37">
+        <v>46181</v>
+      </c>
       <c r="B81" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="C81">
-        <v>344</v>
+        <v>536</v>
       </c>
       <c r="D81">
         <v>4330</v>
       </c>
       <c r="E81">
         <f t="shared" si="1"/>
-        <v>1489520</v>
+        <v>2320880</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
-        <v>517</v>
+        <v>22</v>
       </c>
       <c r="C82">
-        <v>2</v>
+        <v>344</v>
       </c>
       <c r="D82">
         <v>4330</v>
       </c>
       <c r="E82">
         <f t="shared" si="1"/>
-        <v>8660</v>
+        <v>1489520</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
-        <v>19</v>
+        <v>517</v>
       </c>
       <c r="C83">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D83">
         <v>4330</v>
       </c>
       <c r="E83">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>8660</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
-        <v>518</v>
+        <v>19</v>
       </c>
       <c r="C84">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="D84">
         <v>4330</v>
       </c>
       <c r="E84">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
-        <v>101</v>
+        <v>518</v>
       </c>
       <c r="C85">
         <v>550</v>
@@ -21920,70 +21922,70 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
-        <v>330</v>
+        <v>101</v>
       </c>
       <c r="C86">
-        <v>580</v>
+        <v>550</v>
       </c>
       <c r="D86">
         <v>4330</v>
       </c>
       <c r="E86">
         <f t="shared" si="1"/>
-        <v>2511400</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
-        <v>16</v>
+        <v>330</v>
       </c>
       <c r="C87">
-        <v>130</v>
+        <v>580</v>
       </c>
       <c r="D87">
         <v>4330</v>
       </c>
       <c r="E87">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>2511400</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
-        <v>209</v>
+        <v>16</v>
       </c>
       <c r="C88">
-        <v>408</v>
+        <v>130</v>
       </c>
       <c r="D88">
         <v>4330</v>
       </c>
       <c r="E88">
         <f t="shared" si="1"/>
-        <v>1766640</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="37">
-        <v>46182</v>
-      </c>
       <c r="B89" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
       <c r="C89">
-        <v>550</v>
+        <v>408</v>
       </c>
       <c r="D89">
         <v>4330</v>
       </c>
       <c r="E89">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>1766640</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A90" s="37">
+        <v>46182</v>
+      </c>
       <c r="B90" t="s">
-        <v>519</v>
+        <v>183</v>
       </c>
       <c r="C90">
         <v>550</v>
@@ -21998,7 +22000,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
-        <v>62</v>
+        <v>519</v>
       </c>
       <c r="C91">
         <v>550</v>
@@ -22013,7 +22015,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B92" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C92">
         <v>550</v>
@@ -22028,7 +22030,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="C93">
         <v>550</v>
@@ -22043,7 +22045,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="C94">
         <v>550</v>
@@ -22058,283 +22060,283 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
-        <v>148</v>
+        <v>43</v>
       </c>
       <c r="C95">
-        <v>20</v>
+        <v>550</v>
       </c>
       <c r="D95">
         <v>4330</v>
       </c>
       <c r="E95">
         <f t="shared" si="1"/>
-        <v>86600</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
-        <v>95</v>
+        <v>148</v>
       </c>
       <c r="C96">
-        <v>560</v>
+        <v>20</v>
       </c>
       <c r="D96">
         <v>4330</v>
       </c>
       <c r="E96">
         <f t="shared" si="1"/>
-        <v>2424800</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="C97">
-        <v>365</v>
+        <v>560</v>
       </c>
       <c r="D97">
         <v>4330</v>
       </c>
       <c r="E97">
         <f t="shared" si="1"/>
-        <v>1580450</v>
+        <v>2424800</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C98">
-        <v>550</v>
+        <v>365</v>
       </c>
       <c r="D98">
         <v>4330</v>
       </c>
       <c r="E98">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>1580450</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="C99">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D99">
         <v>4330</v>
       </c>
       <c r="E99">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
-        <v>394</v>
+        <v>3</v>
       </c>
       <c r="C100">
-        <v>30</v>
+        <v>130</v>
       </c>
       <c r="D100">
         <v>4330</v>
       </c>
       <c r="E100">
         <f t="shared" si="1"/>
-        <v>129900</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
-        <v>18</v>
+        <v>394</v>
       </c>
       <c r="C101">
-        <v>325</v>
+        <v>30</v>
       </c>
       <c r="D101">
         <v>4330</v>
       </c>
       <c r="E101">
         <f t="shared" si="1"/>
-        <v>1407250</v>
+        <v>129900</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="37">
-        <v>46183</v>
-      </c>
       <c r="B102" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="C102">
-        <v>548</v>
+        <v>325</v>
       </c>
       <c r="D102">
         <v>4330</v>
       </c>
       <c r="E102">
         <f t="shared" si="1"/>
-        <v>2372840</v>
+        <v>1407250</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A103" s="37">
+        <v>46183</v>
+      </c>
       <c r="B103" t="s">
-        <v>520</v>
+        <v>49</v>
       </c>
       <c r="C103">
-        <v>20</v>
+        <v>548</v>
       </c>
       <c r="D103">
         <v>4330</v>
       </c>
       <c r="E103">
         <f t="shared" si="1"/>
-        <v>86600</v>
+        <v>2372840</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
-        <v>19</v>
+        <v>520</v>
       </c>
       <c r="C104">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="D104">
         <v>4330</v>
       </c>
       <c r="E104">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C105">
-        <v>350</v>
+        <v>130</v>
       </c>
       <c r="D105">
         <v>4330</v>
       </c>
       <c r="E105">
         <f t="shared" si="1"/>
-        <v>1515500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
-        <v>521</v>
+        <v>22</v>
       </c>
       <c r="C106">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="D106">
         <v>4330</v>
       </c>
       <c r="E106">
         <f t="shared" si="1"/>
-        <v>86600</v>
+        <v>1515500</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
-        <v>25</v>
+        <v>521</v>
       </c>
       <c r="C107">
-        <v>550</v>
+        <v>20</v>
       </c>
       <c r="D107">
         <v>4330</v>
       </c>
       <c r="E107">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
-        <v>378</v>
+        <v>25</v>
       </c>
       <c r="C108">
-        <v>577</v>
+        <v>550</v>
       </c>
       <c r="D108">
         <v>4330</v>
       </c>
       <c r="E108">
         <f t="shared" si="1"/>
-        <v>2498410</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
-        <v>16</v>
+        <v>378</v>
       </c>
       <c r="C109">
-        <v>130</v>
+        <v>577</v>
       </c>
       <c r="D109">
         <v>4330</v>
       </c>
       <c r="E109">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>2498410</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C110">
-        <v>391</v>
+        <v>130</v>
       </c>
       <c r="D110">
         <v>4330</v>
       </c>
       <c r="E110">
         <f t="shared" si="1"/>
-        <v>1693030</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="37">
-        <v>46184</v>
-      </c>
       <c r="B111" t="s">
-        <v>307</v>
+        <v>26</v>
       </c>
       <c r="C111">
-        <v>580</v>
+        <v>391</v>
       </c>
       <c r="D111">
         <v>4330</v>
       </c>
       <c r="E111">
         <f t="shared" si="1"/>
-        <v>2511400</v>
+        <v>1693030</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A112" s="37">
+        <v>46184</v>
+      </c>
       <c r="B112" t="s">
-        <v>522</v>
+        <v>307</v>
       </c>
       <c r="C112">
-        <v>550</v>
+        <v>580</v>
       </c>
       <c r="D112">
         <v>4330</v>
       </c>
       <c r="E112">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>2511400</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
-        <v>23</v>
+        <v>522</v>
       </c>
       <c r="C113">
         <v>550</v>
@@ -22349,130 +22351,130 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="C114">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D114">
         <v>4330</v>
       </c>
       <c r="E114">
         <f t="shared" si="1"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="C115">
-        <v>376</v>
+        <v>130</v>
       </c>
       <c r="D115">
         <v>4330</v>
       </c>
       <c r="E115">
         <f t="shared" si="1"/>
-        <v>1628080</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C116">
-        <v>550</v>
+        <v>376</v>
       </c>
       <c r="D116">
         <v>4330</v>
       </c>
       <c r="E116">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>1628080</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
-        <v>225</v>
+        <v>115</v>
       </c>
       <c r="C117">
-        <v>575</v>
+        <v>550</v>
       </c>
       <c r="D117">
         <v>4330</v>
       </c>
       <c r="E117">
         <f t="shared" si="1"/>
-        <v>2489750</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="C118">
-        <v>402</v>
+        <v>575</v>
       </c>
       <c r="D118">
         <v>4330</v>
       </c>
       <c r="E118">
         <f t="shared" si="1"/>
-        <v>1740660</v>
+        <v>2489750</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="37">
-        <v>46185</v>
-      </c>
       <c r="B119" t="s">
-        <v>522</v>
+        <v>209</v>
       </c>
       <c r="C119">
-        <v>2</v>
+        <v>402</v>
       </c>
       <c r="D119">
         <v>4330</v>
       </c>
       <c r="E119">
         <f t="shared" si="1"/>
-        <v>8660</v>
+        <v>1740660</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A120" s="37">
+        <v>46185</v>
+      </c>
       <c r="B120" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C120">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D120">
         <v>4330</v>
       </c>
       <c r="E120">
         <f t="shared" si="1"/>
-        <v>43300</v>
+        <v>8660</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
-        <v>210</v>
+        <v>523</v>
       </c>
       <c r="C121">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D121">
         <v>4330</v>
       </c>
       <c r="E121">
         <f t="shared" si="1"/>
-        <v>86600</v>
+        <v>43300</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
-        <v>121</v>
+        <v>210</v>
       </c>
       <c r="C122">
         <v>20</v>
@@ -22487,187 +22489,187 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
-        <v>524</v>
+        <v>121</v>
       </c>
       <c r="C123">
-        <v>570</v>
+        <v>20</v>
       </c>
       <c r="D123">
         <v>4330</v>
       </c>
       <c r="E123">
         <f t="shared" si="1"/>
-        <v>2468100</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C124">
-        <v>585</v>
+        <v>570</v>
       </c>
       <c r="D124">
         <v>4330</v>
       </c>
       <c r="E124">
         <f t="shared" si="1"/>
-        <v>2533050</v>
+        <v>2468100</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
-        <v>172</v>
+        <v>525</v>
       </c>
       <c r="C125">
-        <v>550</v>
+        <v>585</v>
       </c>
       <c r="D125">
         <v>4330</v>
       </c>
       <c r="E125">
         <f t="shared" si="1"/>
-        <v>2381500</v>
+        <v>2533050</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
-        <v>526</v>
+        <v>172</v>
       </c>
       <c r="C126">
-        <v>590</v>
+        <v>550</v>
       </c>
       <c r="D126">
         <v>4330</v>
       </c>
       <c r="E126">
         <f t="shared" si="1"/>
-        <v>2554700</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C127">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="D127">
         <v>4330</v>
       </c>
       <c r="E127">
         <f t="shared" si="1"/>
-        <v>2511400</v>
+        <v>2554700</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
-        <v>49</v>
+        <v>527</v>
       </c>
       <c r="C128">
-        <v>543</v>
+        <v>580</v>
       </c>
       <c r="D128">
         <v>4330</v>
       </c>
       <c r="E128">
         <f t="shared" si="1"/>
-        <v>2351190</v>
+        <v>2511400</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
-        <v>528</v>
+        <v>49</v>
       </c>
       <c r="C129">
-        <v>20</v>
+        <v>543</v>
       </c>
       <c r="D129">
         <v>4330</v>
       </c>
       <c r="E129">
-        <f t="shared" ref="E129:E192" si="2">C129*D129</f>
-        <v>86600</v>
+        <f t="shared" si="1"/>
+        <v>2351190</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
-        <v>149</v>
+        <v>528</v>
       </c>
       <c r="C130">
-        <v>550</v>
+        <v>20</v>
       </c>
       <c r="D130">
         <v>4330</v>
       </c>
       <c r="E130">
-        <f t="shared" si="2"/>
-        <v>2381500</v>
+        <f t="shared" ref="E130:E193" si="2">C130*D130</f>
+        <v>86600</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
-        <v>22</v>
+        <v>149</v>
       </c>
       <c r="C131">
-        <v>357</v>
+        <v>550</v>
       </c>
       <c r="D131">
         <v>4330</v>
       </c>
       <c r="E131">
         <f t="shared" si="2"/>
-        <v>1545810</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
-        <v>528</v>
+        <v>22</v>
       </c>
       <c r="C132">
-        <v>577</v>
+        <v>357</v>
       </c>
       <c r="D132">
         <v>4330</v>
       </c>
       <c r="E132">
         <f t="shared" si="2"/>
-        <v>2498410</v>
+        <v>1545810</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C133">
-        <v>595</v>
+        <v>577</v>
       </c>
       <c r="D133">
         <v>4330</v>
       </c>
       <c r="E133">
         <f t="shared" si="2"/>
-        <v>2576350</v>
+        <v>2498410</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
-        <v>78</v>
+        <v>529</v>
       </c>
       <c r="C134">
-        <v>550</v>
+        <v>595</v>
       </c>
       <c r="D134">
         <v>4330</v>
       </c>
       <c r="E134">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>2576350</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
-        <v>186</v>
+        <v>78</v>
       </c>
       <c r="C135">
         <v>550</v>
@@ -22682,358 +22684,358 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
-        <v>112</v>
+        <v>186</v>
       </c>
       <c r="C136">
-        <v>2</v>
+        <v>550</v>
       </c>
       <c r="D136">
         <v>4330</v>
       </c>
       <c r="E136">
         <f t="shared" si="2"/>
-        <v>8660</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
-        <v>16</v>
+        <v>112</v>
       </c>
       <c r="C137">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D137">
         <v>4330</v>
       </c>
       <c r="E137">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>8660</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
-        <v>521</v>
+        <v>16</v>
       </c>
       <c r="C138">
-        <v>584</v>
+        <v>130</v>
       </c>
       <c r="D138">
         <v>4330</v>
       </c>
       <c r="E138">
         <f t="shared" si="2"/>
-        <v>2528720</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
-        <v>18</v>
+        <v>521</v>
       </c>
       <c r="C139">
-        <v>346</v>
+        <v>584</v>
       </c>
       <c r="D139">
         <v>4330</v>
       </c>
       <c r="E139">
         <f t="shared" si="2"/>
-        <v>1498180</v>
+        <v>2528720</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C140">
-        <v>130</v>
+        <v>346</v>
       </c>
       <c r="D140">
         <v>4330</v>
       </c>
       <c r="E140">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>1498180</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A141" s="37">
-        <v>46186</v>
-      </c>
       <c r="B141" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C141">
-        <v>548</v>
+        <v>130</v>
       </c>
       <c r="D141">
         <v>4330</v>
       </c>
       <c r="E141">
         <f t="shared" si="2"/>
-        <v>2372840</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A142" s="37">
+        <v>46186</v>
+      </c>
       <c r="B142" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="C142">
-        <v>363</v>
+        <v>548</v>
       </c>
       <c r="D142">
         <v>4330</v>
       </c>
       <c r="E142">
         <f t="shared" si="2"/>
-        <v>1571790</v>
+        <v>2372840</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
-        <v>394</v>
+        <v>50</v>
       </c>
       <c r="C143">
-        <v>586</v>
+        <v>363</v>
       </c>
       <c r="D143">
         <v>4330</v>
       </c>
       <c r="E143">
         <f t="shared" si="2"/>
-        <v>2537380</v>
+        <v>1571790</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
-        <v>168</v>
+        <v>394</v>
       </c>
       <c r="C144">
-        <v>20</v>
+        <v>586</v>
       </c>
       <c r="D144">
         <v>4330</v>
       </c>
       <c r="E144">
         <f t="shared" si="2"/>
-        <v>86600</v>
+        <v>2537380</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
-        <v>121</v>
+        <v>168</v>
       </c>
       <c r="C145">
-        <v>580</v>
+        <v>20</v>
       </c>
       <c r="D145">
         <v>4330</v>
       </c>
       <c r="E145">
         <f t="shared" si="2"/>
-        <v>2511400</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
-        <v>3</v>
+        <v>121</v>
       </c>
       <c r="C146">
-        <v>130</v>
+        <v>580</v>
       </c>
       <c r="D146">
         <v>4330</v>
       </c>
       <c r="E146">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>2511400</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="C147">
-        <v>399</v>
+        <v>130</v>
       </c>
       <c r="D147">
         <v>4330</v>
       </c>
       <c r="E147">
         <f t="shared" si="2"/>
-        <v>1727670</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="C148">
-        <v>550</v>
+        <v>399</v>
       </c>
       <c r="D148">
         <v>4330</v>
       </c>
       <c r="E148">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>1727670</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="C149">
-        <v>347</v>
+        <v>550</v>
       </c>
       <c r="D149">
         <v>4330</v>
       </c>
       <c r="E149">
         <f t="shared" si="2"/>
-        <v>1502510</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C150">
-        <v>130</v>
+        <v>347</v>
       </c>
       <c r="D150">
         <v>4330</v>
       </c>
       <c r="E150">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>1502510</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
-        <v>209</v>
+        <v>16</v>
       </c>
       <c r="C151">
-        <v>380</v>
+        <v>130</v>
       </c>
       <c r="D151">
         <v>4330</v>
       </c>
       <c r="E151">
         <f t="shared" si="2"/>
-        <v>1645400</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
-        <v>19</v>
+        <v>209</v>
       </c>
       <c r="C152">
-        <v>130</v>
+        <v>380</v>
       </c>
       <c r="D152">
         <v>4330</v>
       </c>
       <c r="E152">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>1645400</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A153" s="37">
-        <v>46187</v>
-      </c>
       <c r="B153" t="s">
-        <v>239</v>
+        <v>19</v>
       </c>
       <c r="C153">
-        <v>560</v>
+        <v>130</v>
       </c>
       <c r="D153">
         <v>4330</v>
       </c>
       <c r="E153">
         <f t="shared" si="2"/>
-        <v>2424800</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A154" s="37">
+        <v>46187</v>
+      </c>
       <c r="B154" t="s">
-        <v>23</v>
+        <v>239</v>
       </c>
       <c r="C154">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="D154">
         <v>4330</v>
       </c>
       <c r="E154">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>2424800</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
-        <v>530</v>
+        <v>23</v>
       </c>
       <c r="C155">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="D155">
         <v>4330</v>
       </c>
       <c r="E155">
         <f t="shared" si="2"/>
-        <v>2251600</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
-        <v>50</v>
+        <v>530</v>
       </c>
       <c r="C156">
-        <v>333</v>
+        <v>520</v>
       </c>
       <c r="D156">
         <v>4330</v>
       </c>
       <c r="E156">
         <f t="shared" si="2"/>
-        <v>1441890</v>
+        <v>2251600</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
-        <v>531</v>
+        <v>50</v>
       </c>
       <c r="C157">
-        <v>565</v>
+        <v>333</v>
       </c>
       <c r="D157">
         <v>4330</v>
       </c>
       <c r="E157">
         <f t="shared" si="2"/>
-        <v>2446450</v>
+        <v>1441890</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
-        <v>243</v>
+        <v>531</v>
       </c>
       <c r="C158">
-        <v>550</v>
+        <v>565</v>
       </c>
       <c r="D158">
         <v>4330</v>
       </c>
       <c r="E158">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>2446450</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
-        <v>396</v>
+        <v>243</v>
       </c>
       <c r="C159">
         <v>550</v>
@@ -23048,7 +23050,7 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
-        <v>128</v>
+        <v>396</v>
       </c>
       <c r="C160">
         <v>550</v>
@@ -23063,7 +23065,7 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="C161">
         <v>550</v>
@@ -23077,101 +23079,101 @@
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A162" s="37">
-        <v>46190</v>
-      </c>
       <c r="B162" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C162">
-        <v>20</v>
+        <v>550</v>
       </c>
       <c r="D162">
         <v>4330</v>
       </c>
       <c r="E162">
         <f t="shared" si="2"/>
-        <v>86600</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A163" s="37">
+        <v>46190</v>
+      </c>
       <c r="B163" t="s">
-        <v>23</v>
+        <v>122</v>
       </c>
       <c r="C163">
-        <v>550</v>
+        <v>20</v>
       </c>
       <c r="D163">
         <v>4330</v>
       </c>
       <c r="E163">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
-        <v>148</v>
+        <v>23</v>
       </c>
       <c r="C164">
-        <v>465</v>
+        <v>550</v>
       </c>
       <c r="D164">
         <v>4330</v>
       </c>
       <c r="E164">
         <f t="shared" si="2"/>
-        <v>2013450</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
-        <v>299</v>
+        <v>148</v>
       </c>
       <c r="C165">
-        <v>80</v>
+        <v>465</v>
       </c>
       <c r="D165">
         <v>4330</v>
       </c>
       <c r="E165">
         <f t="shared" si="2"/>
-        <v>346400</v>
+        <v>2013450</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
-        <v>22</v>
+        <v>299</v>
       </c>
       <c r="C166">
-        <v>352</v>
+        <v>80</v>
       </c>
       <c r="D166">
         <v>4330</v>
       </c>
       <c r="E166">
         <f t="shared" si="2"/>
-        <v>1524160</v>
+        <v>346400</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C167">
-        <v>550</v>
+        <v>352</v>
       </c>
       <c r="D167">
         <v>4330</v>
       </c>
       <c r="E167">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>1524160</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
-        <v>257</v>
+        <v>45</v>
       </c>
       <c r="C168">
         <v>550</v>
@@ -23186,7 +23188,7 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
-        <v>109</v>
+        <v>257</v>
       </c>
       <c r="C169">
         <v>550</v>
@@ -23201,37 +23203,37 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
-        <v>234</v>
+        <v>109</v>
       </c>
       <c r="C170">
-        <v>437</v>
+        <v>550</v>
       </c>
       <c r="D170">
         <v>4330</v>
       </c>
       <c r="E170">
         <f t="shared" si="2"/>
-        <v>1892210</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
-        <v>123</v>
+        <v>234</v>
       </c>
       <c r="C171">
-        <v>550</v>
+        <v>437</v>
       </c>
       <c r="D171">
         <v>4330</v>
       </c>
       <c r="E171">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>1892210</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C172">
         <v>550</v>
@@ -23246,130 +23248,130 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
-        <v>50</v>
+        <v>133</v>
       </c>
       <c r="C173">
-        <v>365</v>
+        <v>550</v>
       </c>
       <c r="D173">
         <v>4330</v>
       </c>
       <c r="E173">
         <f t="shared" si="2"/>
-        <v>1580450</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="C174">
-        <v>130</v>
+        <v>365</v>
       </c>
       <c r="D174">
         <v>4330</v>
       </c>
       <c r="E174">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>1580450</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
-        <v>209</v>
+        <v>3</v>
       </c>
       <c r="C175">
-        <v>369</v>
+        <v>130</v>
       </c>
       <c r="D175">
         <v>4330</v>
       </c>
       <c r="E175">
         <f t="shared" si="2"/>
-        <v>1597770</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A176" s="37">
-        <v>46191</v>
-      </c>
       <c r="B176" t="s">
-        <v>19</v>
+        <v>209</v>
       </c>
       <c r="C176">
-        <v>130</v>
+        <v>369</v>
       </c>
       <c r="D176">
         <v>4330</v>
       </c>
       <c r="E176">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>1597770</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A177" s="37">
+        <v>46191</v>
+      </c>
       <c r="B177" t="s">
-        <v>194</v>
+        <v>19</v>
       </c>
       <c r="C177">
-        <v>550</v>
+        <v>130</v>
       </c>
       <c r="D177">
         <v>4330</v>
       </c>
       <c r="E177">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
-        <v>122</v>
+        <v>194</v>
       </c>
       <c r="C178">
-        <v>570</v>
+        <v>550</v>
       </c>
       <c r="D178">
         <v>4330</v>
       </c>
       <c r="E178">
         <f t="shared" si="2"/>
-        <v>2468100</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
-        <v>49</v>
+        <v>122</v>
       </c>
       <c r="C179">
-        <v>535</v>
+        <v>570</v>
       </c>
       <c r="D179">
         <v>4330</v>
       </c>
       <c r="E179">
         <f t="shared" si="2"/>
-        <v>2316550</v>
+        <v>2468100</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
-        <v>532</v>
+        <v>49</v>
       </c>
       <c r="C180">
-        <v>550</v>
+        <v>535</v>
       </c>
       <c r="D180">
         <v>4330</v>
       </c>
       <c r="E180">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>2316550</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
-        <v>242</v>
+        <v>532</v>
       </c>
       <c r="C181">
         <v>550</v>
@@ -23384,7 +23386,7 @@
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
-        <v>174</v>
+        <v>242</v>
       </c>
       <c r="C182">
         <v>550</v>
@@ -23399,97 +23401,97 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
-        <v>4</v>
+        <v>174</v>
       </c>
       <c r="C183">
-        <v>343</v>
+        <v>550</v>
       </c>
       <c r="D183">
         <v>4330</v>
       </c>
       <c r="E183">
         <f t="shared" si="2"/>
-        <v>1485190</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
-        <v>392</v>
+        <v>4</v>
       </c>
       <c r="C184">
-        <v>550</v>
+        <v>343</v>
       </c>
       <c r="D184">
         <v>4330</v>
       </c>
       <c r="E184">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>1485190</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
-        <v>533</v>
+        <v>392</v>
       </c>
       <c r="C185">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="D185">
         <v>4330</v>
       </c>
       <c r="E185">
         <f t="shared" si="2"/>
-        <v>2403150</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
-        <v>416</v>
+        <v>533</v>
       </c>
       <c r="C186">
-        <v>20</v>
+        <v>555</v>
       </c>
       <c r="D186">
         <v>4330</v>
       </c>
       <c r="E186">
         <f t="shared" si="2"/>
-        <v>86600</v>
+        <v>2403150</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
-        <v>534</v>
+        <v>416</v>
       </c>
       <c r="C187">
-        <v>556</v>
+        <v>20</v>
       </c>
       <c r="D187">
         <v>4330</v>
       </c>
       <c r="E187">
         <f t="shared" si="2"/>
-        <v>2407480</v>
+        <v>86600</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
-        <v>386</v>
+        <v>534</v>
       </c>
       <c r="C188">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="D188">
         <v>4330</v>
       </c>
       <c r="E188">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>2407480</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
-        <v>329</v>
+        <v>386</v>
       </c>
       <c r="C189">
         <v>550</v>
@@ -23504,55 +23506,55 @@
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
-        <v>16</v>
+        <v>329</v>
       </c>
       <c r="C190">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D190">
         <v>4330</v>
       </c>
       <c r="E190">
         <f t="shared" si="2"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
-        <v>535</v>
+        <v>16</v>
       </c>
       <c r="C191">
-        <v>334</v>
+        <v>130</v>
       </c>
       <c r="D191">
         <v>4330</v>
       </c>
       <c r="E191">
         <f t="shared" si="2"/>
-        <v>1446220</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A192" s="37">
-        <v>46192</v>
-      </c>
       <c r="B192" t="s">
-        <v>23</v>
+        <v>535</v>
       </c>
       <c r="C192">
-        <v>550</v>
+        <v>334</v>
       </c>
       <c r="D192">
         <v>4330</v>
       </c>
       <c r="E192">
         <f t="shared" si="2"/>
-        <v>2381500</v>
+        <v>1446220</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A193" s="37">
+        <v>46192</v>
+      </c>
       <c r="B193" t="s">
-        <v>127</v>
+        <v>23</v>
       </c>
       <c r="C193">
         <v>550</v>
@@ -23561,13 +23563,13 @@
         <v>4330</v>
       </c>
       <c r="E193">
-        <f t="shared" ref="E193:E216" si="3">C193*D193</f>
+        <f t="shared" si="2"/>
         <v>2381500</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
-        <v>151</v>
+        <v>127</v>
       </c>
       <c r="C194">
         <v>550</v>
@@ -23576,73 +23578,73 @@
         <v>4330</v>
       </c>
       <c r="E194">
+        <f t="shared" ref="E194:E217" si="3">C194*D194</f>
+        <v>2381500</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B195" t="s">
+        <v>151</v>
+      </c>
+      <c r="C195">
+        <v>550</v>
+      </c>
+      <c r="D195">
+        <v>4330</v>
+      </c>
+      <c r="E195">
         <f t="shared" si="3"/>
         <v>2381500</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B195" t="s">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B196" t="s">
         <v>22</v>
       </c>
-      <c r="C195">
+      <c r="C196">
         <v>352</v>
       </c>
-      <c r="D195">
+      <c r="D196">
         <v>4330</v>
       </c>
-      <c r="E195">
+      <c r="E196">
         <f t="shared" si="3"/>
         <v>1524160</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B196" t="s">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B197" t="s">
         <v>536</v>
       </c>
-      <c r="C196">
+      <c r="C197">
         <v>20</v>
       </c>
-      <c r="D196">
+      <c r="D197">
         <v>4330</v>
       </c>
-      <c r="E196">
+      <c r="E197">
         <f t="shared" si="3"/>
         <v>86600</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B197" t="s">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B198" t="s">
         <v>287</v>
       </c>
-      <c r="C197">
+      <c r="C198">
         <v>586</v>
       </c>
-      <c r="D197">
+      <c r="D198">
         <v>4330</v>
       </c>
-      <c r="E197">
+      <c r="E198">
         <f t="shared" si="3"/>
         <v>2537380</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B198" t="s">
-        <v>204</v>
-      </c>
-      <c r="C198">
-        <v>550</v>
-      </c>
-      <c r="D198">
-        <v>4330</v>
-      </c>
-      <c r="E198">
-        <f t="shared" si="3"/>
-        <v>2381500</v>
-      </c>
-    </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="C199">
         <v>550</v>
@@ -23657,55 +23659,55 @@
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
-        <v>3</v>
+        <v>80</v>
       </c>
       <c r="C200">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D200">
         <v>4330</v>
       </c>
       <c r="E200">
         <f t="shared" si="3"/>
-        <v>562900</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="C201">
-        <v>373</v>
+        <v>130</v>
       </c>
       <c r="D201">
         <v>4330</v>
       </c>
       <c r="E201">
         <f t="shared" si="3"/>
-        <v>1615090</v>
+        <v>562900</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A202" s="37">
-        <v>46193</v>
-      </c>
       <c r="B202" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C202">
-        <v>2</v>
+        <v>373</v>
       </c>
       <c r="D202">
         <v>4330</v>
       </c>
       <c r="E202">
         <f t="shared" si="3"/>
-        <v>8660</v>
+        <v>1615090</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A203" s="37">
+        <v>46193</v>
+      </c>
       <c r="B203" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C203">
         <v>2</v>
@@ -23720,175 +23722,175 @@
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
-        <v>537</v>
+        <v>24</v>
       </c>
       <c r="C204">
-        <v>555</v>
+        <v>2</v>
       </c>
       <c r="D204">
         <v>4330</v>
       </c>
       <c r="E204">
         <f t="shared" si="3"/>
-        <v>2403150</v>
+        <v>8660</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
-        <v>126</v>
+        <v>537</v>
       </c>
       <c r="C205">
-        <v>575</v>
+        <v>555</v>
       </c>
       <c r="D205">
         <v>4330</v>
       </c>
       <c r="E205">
         <f t="shared" si="3"/>
-        <v>2489750</v>
+        <v>2403150</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
-        <v>49</v>
+        <v>126</v>
       </c>
       <c r="C206">
-        <v>546</v>
+        <v>575</v>
       </c>
       <c r="D206">
         <v>4330</v>
       </c>
       <c r="E206">
         <f t="shared" si="3"/>
-        <v>2364180</v>
+        <v>2489750</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
-        <v>159</v>
+        <v>49</v>
       </c>
       <c r="C207">
-        <v>565</v>
+        <v>546</v>
       </c>
       <c r="D207">
         <v>4330</v>
       </c>
       <c r="E207">
         <f t="shared" si="3"/>
-        <v>2446450</v>
+        <v>2364180</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
-        <v>131</v>
+        <v>159</v>
       </c>
       <c r="C208">
-        <v>550</v>
+        <v>565</v>
       </c>
       <c r="D208">
         <v>4330</v>
       </c>
       <c r="E208">
         <f t="shared" si="3"/>
-        <v>2381500</v>
+        <v>2446450</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
-        <v>351</v>
+        <v>131</v>
       </c>
       <c r="C209">
-        <v>570</v>
+        <v>550</v>
       </c>
       <c r="D209">
         <v>4330</v>
       </c>
       <c r="E209">
         <f t="shared" si="3"/>
-        <v>2468100</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
-        <v>154</v>
+        <v>351</v>
       </c>
       <c r="C210">
-        <v>550</v>
+        <v>570</v>
       </c>
       <c r="D210">
         <v>4330</v>
       </c>
       <c r="E210">
         <f t="shared" si="3"/>
-        <v>2381500</v>
+        <v>2468100</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
-        <v>209</v>
+        <v>154</v>
       </c>
       <c r="C211">
-        <v>363</v>
+        <v>550</v>
       </c>
       <c r="D211">
         <v>4330</v>
       </c>
       <c r="E211">
         <f t="shared" si="3"/>
-        <v>1571790</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
-        <v>23</v>
+        <v>209</v>
       </c>
       <c r="C212">
-        <v>550</v>
+        <v>363</v>
       </c>
       <c r="D212">
         <v>4330</v>
       </c>
       <c r="E212">
         <f t="shared" si="3"/>
-        <v>2381500</v>
+        <v>1571790</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B213" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C213">
-        <v>346</v>
+        <v>550</v>
       </c>
       <c r="D213">
         <v>4330</v>
       </c>
       <c r="E213">
         <f t="shared" si="3"/>
-        <v>1498180</v>
+        <v>2381500</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A214" s="37">
-        <v>46195</v>
-      </c>
       <c r="B214" t="s">
-        <v>145</v>
+        <v>4</v>
       </c>
       <c r="C214">
-        <v>580</v>
+        <v>346</v>
       </c>
       <c r="D214">
         <v>4330</v>
       </c>
       <c r="E214">
         <f t="shared" si="3"/>
-        <v>2511400</v>
+        <v>1498180</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A215" s="37">
+        <v>46195</v>
+      </c>
       <c r="B215" t="s">
-        <v>416</v>
+        <v>145</v>
       </c>
       <c r="C215">
         <v>580</v>
@@ -23903,15 +23905,30 @@
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B216" t="s">
-        <v>108</v>
+        <v>416</v>
       </c>
       <c r="C216">
-        <v>546</v>
+        <v>580</v>
       </c>
       <c r="D216">
         <v>4330</v>
       </c>
       <c r="E216">
+        <f t="shared" si="3"/>
+        <v>2511400</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B217" t="s">
+        <v>108</v>
+      </c>
+      <c r="C217">
+        <v>546</v>
+      </c>
+      <c r="D217">
+        <v>4330</v>
+      </c>
+      <c r="E217">
         <f t="shared" si="3"/>
         <v>2364180</v>
       </c>

</xml_diff>